<commit_message>
fix data driven testing functionality
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -7,19 +7,186 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TopCourses" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LanguageSummary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TestCases" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TestResults" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="33">
+  <si>
+    <t>extractCategoryCatalog</t>
+  </si>
+  <si>
+    <t>RUN_STATUS</t>
+  </si>
+  <si>
+    <t>Expected condition failed: waiting for visibility of element located by By.xpath: //label[@class="ud-heading-xl ud-form-label ud-heading-sm"] (tried for 15 second(s) with 500 milliseconds interval)
+Build info: version: '4.21.0', revision: '79ed462ef4'
+System info: os.name: 'Windows 11', os.arch: 'amd64', os.version: '10.0', java.version: '21.0.10'
+Driver info: org.openqa.selenium.chrome.ChromeDriver
+Capabilities {acceptInsecureCerts: false, browserName: chrome, browserVersion: 149.0.7827.103, chrome: {chromedriverVersion: 149.0.7827.155 (07b52360cc1..., userDataDir: C:\Users\2506400\AppData\Lo...}, fedcm:accounts: true, goog:chromeOptions: {debuggerAddress: localhost:56244}, goog:processID: 18996, networkConnectionEnabled: false, pageLoadStrategy: normal, platformName: windows, proxy: Proxy(), se:cdp: ws://localhost:56244/devtoo..., se:cdpVersion: 149.0.7827.103, setWindowRect: true, strictFileInteractability: false, timeouts: {implicit: 0, pageLoad: 300000, script: 30000}, unhandledPromptBehavior: dismiss and notify, webauthn:extension:credBlob: true, webauthn:extension:largeBlob: true, webauthn:extension:minPinLength: true, webauthn:extension:prf: true, webauthn:virtualAuthenticators: true}
+Session ID: 66528ef8bd9949cf01781d771eb21206</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>FAIL</t>
+  </si>
+  <si>
+    <t>2026-07-20 17:28:58</t>
+  </si>
+  <si>
+    <t>Expected condition failed: waiting for visibility of element located by By.xpath: //label[@class="ud-heading-xl ud-form-label ud-heading-sm"] (tried for 15 second(s) with 500 milliseconds interval)
+Build info: version: '4.21.0', revision: '79ed462ef4'
+System info: os.name: 'Windows 11', os.arch: 'amd64', os.version: '10.0', java.version: '21.0.10'
+Driver info: org.openqa.selenium.chrome.ChromeDriver
+Capabilities {acceptInsecureCerts: false, browserName: chrome, browserVersion: 149.0.7827.103, chrome: {chromedriverVersion: 149.0.7827.155 (07b52360cc1..., userDataDir: C:\Users\2506400\AppData\Lo...}, fedcm:accounts: true, goog:chromeOptions: {debuggerAddress: localhost:57957}, goog:processID: 29184, networkConnectionEnabled: false, pageLoadStrategy: normal, platformName: windows, proxy: Proxy(), se:cdp: ws://localhost:57957/devtoo..., se:cdpVersion: 149.0.7827.103, setWindowRect: true, strictFileInteractability: false, timeouts: {implicit: 0, pageLoad: 300000, script: 30000}, unhandledPromptBehavior: dismiss and notify, webauthn:extension:credBlob: true, webauthn:extension:largeBlob: true, webauthn:extension:minPinLength: true, webauthn:extension:prf: true, webauthn:virtualAuthenticators: true}
+Session ID: 0325edcc662cee1c30c1c27c577cfe0e</t>
+  </si>
+  <si>
+    <t>2026-07-20 17:35:34</t>
+  </si>
+  <si>
+    <t>Expected condition failed: waiting for visibility of element located by By.xpath: //*[normalize-space(text())='Language'] (tried for 15 second(s) with 500 milliseconds interval)
+Build info: version: '4.21.0', revision: '79ed462ef4'
+System info: os.name: 'Windows 11', os.arch: 'amd64', os.version: '10.0', java.version: '21.0.10'
+Driver info: org.openqa.selenium.chrome.ChromeDriver
+Capabilities {acceptInsecureCerts: false, browserName: chrome, browserVersion: 149.0.7827.103, chrome: {chromedriverVersion: 149.0.7827.155 (07b52360cc1..., userDataDir: C:\Users\2506400\AppData\Lo...}, fedcm:accounts: true, goog:chromeOptions: {debuggerAddress: localhost:63310}, goog:processID: 27376, networkConnectionEnabled: false, pageLoadStrategy: normal, platformName: windows, proxy: Proxy(), se:cdp: ws://localhost:63310/devtoo..., se:cdpVersion: 149.0.7827.103, setWindowRect: true, strictFileInteractability: false, timeouts: {implicit: 0, pageLoad: 300000, script: 30000}, unhandledPromptBehavior: dismiss and notify, webauthn:extension:credBlob: true, webauthn:extension:largeBlob: true, webauthn:extension:minPinLength: true, webauthn:extension:prf: true, webauthn:virtualAuthenticators: true}
+Session ID: adf65a615c8136ef553c30163775d80c</t>
+  </si>
+  <si>
+    <t>2026-07-20 19:08:32</t>
+  </si>
+  <si>
+    <t>Expected condition failed: waiting for visibility of element located by By.xpath: //*[normalize-space(text())='Language'] (tried for 15 second(s) with 500 milliseconds interval)
+Build info: version: '4.21.0', revision: '79ed462ef4'
+System info: os.name: 'Windows 11', os.arch: 'amd64', os.version: '10.0', java.version: '21.0.10'
+Driver info: org.openqa.selenium.chrome.ChromeDriver
+Capabilities {acceptInsecureCerts: false, browserName: chrome, browserVersion: 149.0.7827.103, chrome: {chromedriverVersion: 149.0.7827.155 (07b52360cc1..., userDataDir: C:\Users\2506400\AppData\Lo...}, fedcm:accounts: true, goog:chromeOptions: {debuggerAddress: localhost:50944}, goog:processID: 11336, networkConnectionEnabled: false, pageLoadStrategy: normal, platformName: windows, proxy: Proxy(), se:cdp: ws://localhost:50944/devtoo..., se:cdpVersion: 149.0.7827.103, setWindowRect: true, strictFileInteractability: false, timeouts: {implicit: 0, pageLoad: 300000, script: 30000}, unhandledPromptBehavior: dismiss and notify, webauthn:extension:credBlob: true, webauthn:extension:largeBlob: true, webauthn:extension:minPinLength: true, webauthn:extension:prf: true, webauthn:virtualAuthenticators: true}
+Session ID: f5fec3ddb48472c244316b5a21a25c41</t>
+  </si>
+  <si>
+    <t>2026-07-20 19:23:53</t>
+  </si>
+  <si>
+    <t>TC_01</t>
+  </si>
+  <si>
+    <t>Expected condition failed: waiting for visibility of element located by By.xpath: //label[contains(@class,'ud-toggle-input-container') and contains(.,'Beginner')] (tried for 15 second(s) with 500 milliseconds interval)
+Build info: version: '4.21.0', revision: '79ed462ef4'
+System info: os.name: 'Windows 11', os.arch: 'amd64', os.version: '10.0', java.version: '21.0.10'
+Driver info: org.openqa.selenium.chrome.ChromeDriver
+Capabilities {acceptInsecureCerts: false, browserName: chrome, browserVersion: 149.0.7827.103, chrome: {chromedriverVersion: 149.0.7827.155 (07b52360cc1..., userDataDir: C:\Users\2506400\AppData\Lo...}, fedcm:accounts: true, goog:chromeOptions: {debuggerAddress: localhost:53297}, goog:processID: 22564, networkConnectionEnabled: false, pageLoadStrategy: normal, platformName: windows, proxy: Proxy(), se:cdp: ws://localhost:53297/devtoo..., se:cdpVersion: 149.0.7827.103, setWindowRect: true, strictFileInteractability: false, timeouts: {implicit: 0, pageLoad: 300000, script: 30000}, unhandledPromptBehavior: dismiss and notify, webauthn:extension:credBlob: true, webauthn:extension:largeBlob: true, webauthn:extension:minPinLength: true, webauthn:extension:prf: true, webauthn:virtualAuthenticators: true}
+Session ID: 48a674e183ca16b3558f8a5f90e441d2</t>
+  </si>
+  <si>
+    <t>2026-07-21 09:44:11</t>
+  </si>
+  <si>
+    <t>TC_02</t>
+  </si>
+  <si>
+    <t>Expected condition failed: waiting for visibility of element located by By.xpath: //label[contains(@class,'ud-toggle-input-container') and contains(.,'Beginner')] (tried for 15 second(s) with 500 milliseconds interval)
+Build info: version: '4.21.0', revision: '79ed462ef4'
+System info: os.name: 'Windows 11', os.arch: 'amd64', os.version: '10.0', java.version: '21.0.10'
+Driver info: org.openqa.selenium.chrome.ChromeDriver
+Capabilities {acceptInsecureCerts: false, browserName: chrome, browserVersion: 149.0.7827.103, chrome: {chromedriverVersion: 149.0.7827.155 (07b52360cc1..., userDataDir: C:\Users\2506400\AppData\Lo...}, fedcm:accounts: true, goog:chromeOptions: {debuggerAddress: localhost:56232}, goog:processID: 11552, networkConnectionEnabled: false, pageLoadStrategy: normal, platformName: windows, proxy: Proxy(), se:cdp: ws://localhost:56232/devtoo..., se:cdpVersion: 149.0.7827.103, setWindowRect: true, strictFileInteractability: false, timeouts: {implicit: 0, pageLoad: 300000, script: 30000}, unhandledPromptBehavior: dismiss and notify, webauthn:extension:credBlob: true, webauthn:extension:largeBlob: true, webauthn:extension:minPinLength: true, webauthn:extension:prf: true, webauthn:virtualAuthenticators: true}
+Session ID: 55009abc805d38331e7d22396922d65c</t>
+  </si>
+  <si>
+    <t>2026-07-21 09:44:47</t>
+  </si>
+  <si>
+    <t>TC_03</t>
+  </si>
+  <si>
+    <t>Expected condition failed: waiting for visibility of element located by By.xpath: //label[contains(@class,'ud-toggle-input-container') and contains(.,'Intermediate')] (tried for 15 second(s) with 500 milliseconds interval)
+Build info: version: '4.21.0', revision: '79ed462ef4'
+System info: os.name: 'Windows 11', os.arch: 'amd64', os.version: '10.0', java.version: '21.0.10'
+Driver info: org.openqa.selenium.chrome.ChromeDriver
+Capabilities {acceptInsecureCerts: false, browserName: chrome, browserVersion: 149.0.7827.103, chrome: {chromedriverVersion: 149.0.7827.155 (07b52360cc1..., userDataDir: C:\Users\2506400\AppData\Lo...}, fedcm:accounts: true, goog:chromeOptions: {debuggerAddress: localhost:62519}, goog:processID: 15228, networkConnectionEnabled: false, pageLoadStrategy: normal, platformName: windows, proxy: Proxy(), se:cdp: ws://localhost:62519/devtoo..., se:cdpVersion: 149.0.7827.103, setWindowRect: true, strictFileInteractability: false, timeouts: {implicit: 0, pageLoad: 300000, script: 30000}, unhandledPromptBehavior: dismiss and notify, webauthn:extension:credBlob: true, webauthn:extension:largeBlob: true, webauthn:extension:minPinLength: true, webauthn:extension:prf: true, webauthn:virtualAuthenticators: true}
+Session ID: 6ba67732f6a968729cf4e5d258932bfc</t>
+  </si>
+  <si>
+    <t>2026-07-21 09:45:23</t>
+  </si>
+  <si>
+    <t>Expected condition failed: waiting for visibility of element located by By.xpath: //*[normalize-space(text())='Language'] (tried for 15 second(s) with 500 milliseconds interval)
+Build info: version: '4.21.0', revision: '79ed462ef4'
+System info: os.name: 'Windows 11', os.arch: 'amd64', os.version: '10.0', java.version: '21.0.10'
+Driver info: org.openqa.selenium.chrome.ChromeDriver
+Capabilities {acceptInsecureCerts: false, browserName: chrome, browserVersion: 149.0.7827.103, chrome: {chromedriverVersion: 149.0.7827.155 (07b52360cc1..., userDataDir: C:\Users\2506400\AppData\Lo...}, fedcm:accounts: true, goog:chromeOptions: {debuggerAddress: localhost:62215}, goog:processID: 2108, networkConnectionEnabled: false, pageLoadStrategy: normal, platformName: windows, proxy: Proxy(), se:cdp: ws://localhost:62215/devtoo..., se:cdpVersion: 149.0.7827.103, setWindowRect: true, strictFileInteractability: false, timeouts: {implicit: 0, pageLoad: 300000, script: 30000}, unhandledPromptBehavior: dismiss and notify, webauthn:extension:credBlob: true, webauthn:extension:largeBlob: true, webauthn:extension:minPinLength: true, webauthn:extension:prf: true, webauthn:virtualAuthenticators: true}
+Session ID: 1526c559699c719d7c85d082e36142c8</t>
+  </si>
+  <si>
+    <t>2026-07-21 09:46:07</t>
+  </si>
+  <si>
+    <t>Expected condition failed: waiting for visibility of element located by By.xpath: //*[normalize-space(text())='Language'] (tried for 15 second(s) with 500 milliseconds interval)
+Build info: version: '4.21.0', revision: '79ed462ef4'
+System info: os.name: 'Windows 11', os.arch: 'amd64', os.version: '10.0', java.version: '21.0.10'
+Driver info: org.openqa.selenium.chrome.ChromeDriver
+Capabilities {acceptInsecureCerts: false, browserName: chrome, browserVersion: 149.0.7827.103, chrome: {chromedriverVersion: 149.0.7827.155 (07b52360cc1..., userDataDir: C:\Users\2506400\AppData\Lo...}, fedcm:accounts: true, goog:chromeOptions: {debuggerAddress: localhost:56648}, goog:processID: 25152, networkConnectionEnabled: false, pageLoadStrategy: normal, platformName: windows, proxy: Proxy(), se:cdp: ws://localhost:56648/devtoo..., se:cdpVersion: 149.0.7827.103, setWindowRect: true, strictFileInteractability: false, timeouts: {implicit: 0, pageLoad: 300000, script: 30000}, unhandledPromptBehavior: dismiss and notify, webauthn:extension:credBlob: true, webauthn:extension:largeBlob: true, webauthn:extension:minPinLength: true, webauthn:extension:prf: true, webauthn:virtualAuthenticators: true}
+Session ID: 227ec593e907c9ab6ec03b0e7c894307</t>
+  </si>
+  <si>
+    <t>2026-07-21 09:46:45</t>
+  </si>
+  <si>
+    <t>Expected condition failed: waiting for visibility of element located by By.xpath: //*[normalize-space(text())='Language'] (tried for 15 second(s) with 500 milliseconds interval)
+Build info: version: '4.21.0', revision: '79ed462ef4'
+System info: os.name: 'Windows 11', os.arch: 'amd64', os.version: '10.0', java.version: '21.0.10'
+Driver info: org.openqa.selenium.chrome.ChromeDriver
+Capabilities {acceptInsecureCerts: false, browserName: chrome, browserVersion: 149.0.7827.103, chrome: {chromedriverVersion: 149.0.7827.155 (07b52360cc1..., userDataDir: C:\Users\2506400\AppData\Lo...}, fedcm:accounts: true, goog:chromeOptions: {debuggerAddress: localhost:61476}, goog:processID: 19648, networkConnectionEnabled: false, pageLoadStrategy: normal, platformName: windows, proxy: Proxy(), se:cdp: ws://localhost:61476/devtoo..., se:cdpVersion: 149.0.7827.103, setWindowRect: true, strictFileInteractability: false, timeouts: {implicit: 0, pageLoad: 300000, script: 30000}, unhandledPromptBehavior: dismiss and notify, webauthn:extension:credBlob: true, webauthn:extension:largeBlob: true, webauthn:extension:minPinLength: true, webauthn:extension:prf: true, webauthn:virtualAuthenticators: true}
+Session ID: ddcfc70a98d2de07ed25e88504f24cb2</t>
+  </si>
+  <si>
+    <t>2026-07-21 09:47:20</t>
+  </si>
+  <si>
+    <t>Expected condition failed: waiting for element to be clickable: By.xpath: //a[@class="section-header single btn-get-started"] (tried for 15 second(s) with 500 milliseconds interval)
+Build info: version: '4.21.0', revision: '79ed462ef4'
+System info: os.name: 'Windows 11', os.arch: 'amd64', os.version: '10.0', java.version: '21.0.10'
+Driver info: org.openqa.selenium.chrome.ChromeDriver
+Capabilities {acceptInsecureCerts: false, browserName: chrome, browserVersion: 149.0.7827.103, chrome: {chromedriverVersion: 149.0.7827.155 (07b52360cc1..., userDataDir: C:\Users\2506400\AppData\Lo...}, fedcm:accounts: true, goog:chromeOptions: {debuggerAddress: localhost:61491}, goog:processID: 15632, networkConnectionEnabled: false, pageLoadStrategy: normal, platformName: windows, proxy: Proxy(), se:cdp: ws://localhost:61491/devtoo..., se:cdpVersion: 149.0.7827.103, setWindowRect: true, strictFileInteractability: false, timeouts: {implicit: 0, pageLoad: 300000, script: 30000}, unhandledPromptBehavior: dismiss and notify, webauthn:extension:credBlob: true, webauthn:extension:largeBlob: true, webauthn:extension:minPinLength: true, webauthn:extension:prf: true, webauthn:virtualAuthenticators: true}
+Session ID: 576f5f2561b6215165a777fc16ee0b9f</t>
+  </si>
+  <si>
+    <t>2026-07-21 09:48:04</t>
+  </si>
+  <si>
+    <t>Expected condition failed: waiting for js return document.readyState==='complete' to be executable (tried for 10 second(s) with 500 milliseconds interval)
+Build info: version: '4.21.0', revision: '79ed462ef4'
+System info: os.name: 'Windows 11', os.arch: 'amd64', os.version: '10.0', java.version: '21.0.10'
+Driver info: org.openqa.selenium.chrome.ChromeDriver
+Capabilities {acceptInsecureCerts: false, browserName: chrome, browserVersion: 149.0.7827.103, chrome: {chromedriverVersion: 149.0.7827.155 (07b52360cc1..., userDataDir: C:\Users\2506400\AppData\Lo...}, fedcm:accounts: true, goog:chromeOptions: {debuggerAddress: localhost:52530}, goog:processID: 13828, networkConnectionEnabled: false, pageLoadStrategy: normal, platformName: windows, proxy: Proxy(), se:cdp: ws://localhost:52530/devtoo..., se:cdpVersion: 149.0.7827.103, setWindowRect: true, strictFileInteractability: false, timeouts: {implicit: 0, pageLoad: 300000, script: 30000}, unhandledPromptBehavior: dismiss and notify, webauthn:extension:credBlob: true, webauthn:extension:largeBlob: true, webauthn:extension:minPinLength: true, webauthn:extension:prf: true, webauthn:virtualAuthenticators: true}
+Session ID: c2406bf0bef9dbdb89b620e40750fa61</t>
+  </si>
+  <si>
+    <t>2026-07-21 09:48:31</t>
+  </si>
+  <si>
+    <t>Expected condition failed: waiting for element to be clickable: By.xpath: //a[@class="section-header single btn-get-started"] (tried for 15 second(s) with 500 milliseconds interval)
+Build info: version: '4.21.0', revision: '79ed462ef4'
+System info: os.name: 'Windows 11', os.arch: 'amd64', os.version: '10.0', java.version: '21.0.10'
+Driver info: org.openqa.selenium.chrome.ChromeDriver
+Capabilities {acceptInsecureCerts: false, browserName: chrome, browserVersion: 149.0.7827.103, chrome: {chromedriverVersion: 149.0.7827.155 (07b52360cc1..., userDataDir: C:\Users\2506400\AppData\Lo...}, fedcm:accounts: true, goog:chromeOptions: {debuggerAddress: localhost:55416}, goog:processID: 25164, networkConnectionEnabled: false, pageLoadStrategy: normal, platformName: windows, proxy: Proxy(), se:cdp: ws://localhost:55416/devtoo..., se:cdpVersion: 149.0.7827.103, setWindowRect: true, strictFileInteractability: false, timeouts: {implicit: 0, pageLoad: 300000, script: 30000}, unhandledPromptBehavior: dismiss and notify, webauthn:extension:credBlob: true, webauthn:extension:largeBlob: true, webauthn:extension:minPinLength: true, webauthn:extension:prf: true, webauthn:virtualAuthenticators: true}
+Session ID: afdb9369b9b44dd517cf91c45141bdd3</t>
+  </si>
+  <si>
+    <t>2026-07-21 09:49:08</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,20 +195,17 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
     <font>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <i val="1"/>
-      <sz val="9"/>
+      <name val="Calibri"/>
+      <sz val="11"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -50,14 +214,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00305496"/>
-        <bgColor rgb="00305496"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
-        <bgColor rgb="00FFFF00"/>
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
       </patternFill>
     </fill>
   </fills>
@@ -73,12 +231,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -444,75 +600,184 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col min="1" max="1" customWidth="true" width="12.0"/>
+    <col min="2" max="2" customWidth="true" width="22.0"/>
+    <col min="3" max="3" customWidth="true" width="14.0"/>
+    <col min="4" max="4" customWidth="true" width="16.0"/>
+    <col min="5" max="5" customWidth="true" width="14.0"/>
+    <col min="6" max="6" customWidth="true" width="14.0"/>
+    <col min="7" max="7" customWidth="true" width="26.0"/>
+    <col min="8" max="8" customWidth="true" width="14.0"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Key</t>
+          <t>TestCaseID</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Legend: yellow cells are the editable inputs read by ExcelUtils.readConfigSheet() / config.properties.</t>
+          <t>Keyword</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>LevelFilter</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>LanguageFilter</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>FirstName</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>LastName</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>WorkEmail</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Phone</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>searchKeyword</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>TC_01</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>web development</t>
         </is>
       </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Beginner</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Aisha</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Khan</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>aisha.khan@@test.com</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>9876543210</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>invalidEmail</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>notarealemail@@com</t>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>TC_02</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>python programming</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Beginner</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Rohan</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Verma</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>rohanvermaatgmail.com</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>9876543211</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>categoryFilterGroup</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Language</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>topCoursesCount</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>TC_03</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>data science</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Intermediate</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Neha</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Sharma</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>neha.sharma@nodomain</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>9876543212</t>
         </is>
       </c>
     </row>
@@ -527,69 +792,352 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col min="1" max="1" customWidth="true" width="12.0"/>
+    <col min="2" max="2" customWidth="true" width="12.0"/>
+    <col min="3" max="3" customWidth="true" width="30.0"/>
+    <col min="4" max="4" customWidth="true" width="14.0"/>
+    <col min="5" max="5" customWidth="true" width="12.0"/>
+    <col min="6" max="6" customWidth="true" width="10.0"/>
+    <col min="7" max="7" customWidth="true" width="18.0"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Course Name</t>
+          <t>TestCaseID</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Duration</t>
+          <t>Type</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Rating</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>Auto-populated by ExcelUtils.writeCourseResults() after IdentifyCoursesTest runs. Leave empty.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Filter Option</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Course Count</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Auto-populated by ExcelUtils.writeCategorySummary() after CategoryExtractionTest runs. Leave empty.</t>
-        </is>
+          <t>Detail1</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Detail2</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Detail3</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Timestamp</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>2</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="G2" t="s" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F3" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="G3" t="s" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F4" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="G4" t="s" s="0">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F5" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="G5" t="s" s="0">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F6" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="G6" t="s" s="0">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E7" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F7" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="G7" t="s" s="0">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="D8" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E8" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F8" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="G8" t="s" s="0">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="D9" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E9" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F9" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="G9" t="s" s="0">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C10" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="D10" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E10" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F10" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="G10" t="s" s="0">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C11" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="D11" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E11" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F11" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="G11" t="s" s="0">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C12" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="D12" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E12" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F12" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="G12" t="s" s="0">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C13" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="D13" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E13" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F13" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="G13" t="s" s="0">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B14" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="D14" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E14" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F14" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="G14" t="s" s="0">
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
remove capture hover message functionality
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -3,9 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{D8A9C4DA-007F-41EE-81E8-DEA551A1550C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2506400\Desktop\Pooja-Workspace\UdemyAutomation\src\test\resources\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FD8CA22-8FA5-41C1-8353-5107B9FB4836}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TestCases" sheetId="1" r:id="rId1"/>
@@ -13,7 +18,6 @@
     <sheet name="TestResults" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="D1:O6"/>
   <extLst>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="2"/>
@@ -23,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="533" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="530" uniqueCount="200">
   <si>
     <t>extractCategoryCatalog</t>
   </si>
@@ -643,9 +647,6 @@
   </si>
   <si>
     <t>Course Publisher</t>
-  </si>
-  <si>
-    <t>Message Captured On Hover</t>
   </si>
   <si>
     <t>CompanyName</t>
@@ -866,7 +867,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1241,23 +1241,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U8"/>
+  <dimension ref="A1:U7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="12.0"/>
-    <col min="2" max="2" customWidth="true" width="22.0"/>
-    <col min="3" max="3" customWidth="true" width="14.0"/>
-    <col min="4" max="4" customWidth="true" width="16.0"/>
-    <col min="5" max="6" customWidth="true" width="14.0"/>
-    <col min="7" max="7" customWidth="true" width="22.6328125"/>
-    <col min="8" max="8" customWidth="true" width="14.90625"/>
-    <col min="9" max="14" customWidth="true" hidden="true" width="8.7265625"/>
-    <col min="15" max="15" customWidth="true" width="21.36328125"/>
-    <col min="16" max="16" customWidth="true" width="17.81640625"/>
-    <col min="17" max="17" customWidth="true" width="20.6328125"/>
-    <col min="18" max="18" customWidth="true" width="21.81640625"/>
-    <col min="19" max="20" customWidth="true" width="15.7265625"/>
-    <col min="21" max="21" customWidth="true" width="59.6328125"/>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="6" width="14" customWidth="1"/>
+    <col min="7" max="7" width="22.6328125" customWidth="1"/>
+    <col min="8" max="8" width="14.90625" customWidth="1"/>
+    <col min="9" max="14" width="8.7265625" hidden="1" customWidth="1"/>
+    <col min="15" max="15" width="21.36328125" customWidth="1"/>
+    <col min="16" max="16" width="17.81640625" customWidth="1"/>
+    <col min="17" max="17" width="20.6328125" customWidth="1"/>
+    <col min="18" max="18" width="21.81640625" customWidth="1"/>
+    <col min="19" max="20" width="15.7265625" customWidth="1"/>
+    <col min="21" max="21" width="59.6328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.35">
@@ -1265,7 +1265,7 @@
         <v>102</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>103</v>
@@ -1283,10 +1283,10 @@
         <v>107</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
@@ -1294,25 +1294,25 @@
       <c r="M1" s="1"/>
       <c r="N1" s="1"/>
       <c r="O1" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="P1" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="Q1" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="Q1" s="4" t="s">
+      <c r="R1" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="R1" s="4" t="s">
+      <c r="S1" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="S1" s="4" t="s">
-        <v>162</v>
-      </c>
       <c r="T1" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="U1" s="4" t="s">
         <v>138</v>
-      </c>
-      <c r="U1" s="4" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.35">
@@ -1337,30 +1337,30 @@
       <c r="G2" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="H2" t="s" s="0">
+      <c r="H2" t="s">
+        <v>139</v>
+      </c>
+      <c r="I2" s="3"/>
+      <c r="O2" t="s">
         <v>140</v>
       </c>
-      <c r="I2" s="3"/>
-      <c r="O2" t="s" s="0">
+      <c r="P2" t="s">
         <v>141</v>
       </c>
-      <c r="P2" t="s" s="0">
+      <c r="Q2" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="R2" t="s">
+        <v>162</v>
+      </c>
+      <c r="S2" t="s">
+        <v>163</v>
+      </c>
+      <c r="T2" t="s">
         <v>142</v>
       </c>
-      <c r="Q2" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="R2" t="s" s="0">
-        <v>163</v>
-      </c>
-      <c r="S2" t="s" s="0">
-        <v>164</v>
-      </c>
-      <c r="T2" t="s" s="0">
+      <c r="U2" t="s">
         <v>143</v>
-      </c>
-      <c r="U2" t="s" s="0">
-        <v>144</v>
       </c>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.35">
@@ -1385,30 +1385,30 @@
       <c r="G3" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="H3" t="s" s="0">
+      <c r="H3" t="s">
+        <v>148</v>
+      </c>
+      <c r="I3" s="3"/>
+      <c r="O3" t="s">
+        <v>147</v>
+      </c>
+      <c r="P3" t="s">
+        <v>146</v>
+      </c>
+      <c r="Q3" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="I3" s="3"/>
-      <c r="O3" t="s" s="0">
-        <v>148</v>
-      </c>
-      <c r="P3" t="s" s="0">
-        <v>147</v>
-      </c>
-      <c r="Q3" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="R3" t="s" s="0">
+      <c r="R3" t="s">
+        <v>164</v>
+      </c>
+      <c r="S3" t="s">
         <v>165</v>
       </c>
-      <c r="S3" t="s" s="0">
-        <v>166</v>
-      </c>
-      <c r="T3" t="s" s="0">
-        <v>146</v>
-      </c>
-      <c r="U3" t="s" s="0">
+      <c r="T3" t="s">
         <v>145</v>
+      </c>
+      <c r="U3" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.35">
@@ -1433,30 +1433,30 @@
       <c r="G4" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="H4" t="s" s="0">
+      <c r="H4" t="s">
+        <v>151</v>
+      </c>
+      <c r="I4" s="3"/>
+      <c r="O4" t="s">
+        <v>168</v>
+      </c>
+      <c r="P4" t="s">
         <v>152</v>
       </c>
-      <c r="I4" s="3"/>
-      <c r="O4" t="s" s="0">
-        <v>169</v>
-      </c>
-      <c r="P4" t="s" s="0">
+      <c r="Q4" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="R4" t="s">
+        <v>166</v>
+      </c>
+      <c r="S4" t="s">
+        <v>167</v>
+      </c>
+      <c r="T4" t="s">
         <v>153</v>
       </c>
-      <c r="Q4" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="R4" t="s" s="0">
-        <v>167</v>
-      </c>
-      <c r="S4" t="s" s="0">
-        <v>168</v>
-      </c>
-      <c r="T4" t="s" s="0">
+      <c r="U4" t="s">
         <v>154</v>
-      </c>
-      <c r="U4" t="s" s="0">
-        <v>155</v>
       </c>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.35">
@@ -1468,7 +1468,6 @@
     <row r="7" spans="1:21" x14ac:dyDescent="0.35">
       <c r="I7" s="3"/>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.35"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -1477,19 +1476,19 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88BFA3FA-6A41-46D8-9F46-57C4912E9286}">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="14.08984375"/>
-    <col min="3" max="3" customWidth="true" width="19.08984375"/>
-    <col min="4" max="4" customWidth="true" width="8.7265625"/>
-    <col min="5" max="5" customWidth="true" width="17.7265625"/>
-    <col min="6" max="6" customWidth="true" width="14.54296875"/>
-    <col min="7" max="7" customWidth="true" width="15.7265625"/>
-    <col min="8" max="8" customWidth="true" width="29.36328125"/>
+    <col min="1" max="1" width="14.08984375" customWidth="1"/>
+    <col min="2" max="2" width="19.453125" customWidth="1"/>
+    <col min="3" max="3" width="19.08984375" customWidth="1"/>
+    <col min="4" max="4" width="8.7265625" customWidth="1"/>
+    <col min="5" max="5" width="17.7265625" customWidth="1"/>
+    <col min="6" max="6" width="14.54296875" customWidth="1"/>
+    <col min="7" max="7" width="15.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>102</v>
       </c>
@@ -1511,60 +1510,51 @@
       <c r="G1" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s" s="0">
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>15</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s">
+        <v>179</v>
+      </c>
+      <c r="C2" t="s">
         <v>180</v>
       </c>
-      <c r="C2" t="s" s="0">
-        <v>181</v>
-      </c>
-      <c r="D2" t="s" s="0">
-        <v>177</v>
-      </c>
-      <c r="E2" t="s" s="0">
-        <v>177</v>
-      </c>
-      <c r="F2" t="s" s="0">
-        <v>177</v>
-      </c>
-      <c r="G2" t="s" s="0">
-        <v>177</v>
-      </c>
-      <c r="H2" t="s" s="0">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s" s="0">
+      <c r="D2" t="s">
+        <v>176</v>
+      </c>
+      <c r="E2" t="s">
+        <v>176</v>
+      </c>
+      <c r="F2" t="s">
+        <v>176</v>
+      </c>
+      <c r="G2" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>18</v>
       </c>
-      <c r="B3" t="s" s="0">
+      <c r="B3" t="s">
+        <v>191</v>
+      </c>
+      <c r="C3" t="s">
         <v>192</v>
       </c>
-      <c r="C3" t="s" s="0">
-        <v>193</v>
-      </c>
-      <c r="D3" t="s" s="0">
-        <v>177</v>
-      </c>
-      <c r="E3" t="s" s="0">
-        <v>177</v>
-      </c>
-      <c r="F3" t="s" s="0">
-        <v>177</v>
-      </c>
-      <c r="G3" t="s" s="0">
-        <v>177</v>
-      </c>
-      <c r="H3" t="s" s="0">
-        <v>3</v>
+      <c r="D3" t="s">
+        <v>176</v>
+      </c>
+      <c r="E3" t="s">
+        <v>176</v>
+      </c>
+      <c r="F3" t="s">
+        <v>176</v>
+      </c>
+      <c r="G3" t="s">
+        <v>176</v>
       </c>
     </row>
   </sheetData>
@@ -1577,12 +1567,12 @@
   <dimension ref="A1:G64"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" customWidth="true" width="12.0"/>
-    <col min="3" max="3" customWidth="true" width="30.0"/>
-    <col min="4" max="4" customWidth="true" width="14.0"/>
-    <col min="5" max="5" customWidth="true" width="12.0"/>
-    <col min="6" max="6" customWidth="true" width="10.0"/>
-    <col min="7" max="7" customWidth="true" width="18.0"/>
+    <col min="1" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="30" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="6" max="6" width="10" customWidth="1"/>
+    <col min="7" max="7" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
@@ -1609,1452 +1599,1452 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C2" t="s" s="0">
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
         <v>2</v>
       </c>
-      <c r="D2" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E2" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F2" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G2" t="s" s="0">
+      <c r="D2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3" t="s" s="0">
+      <c r="A3" t="s">
         <v>0</v>
       </c>
-      <c r="B3" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C3" t="s" s="0">
+      <c r="B3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
         <v>6</v>
       </c>
-      <c r="D3" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E3" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F3" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G3" t="s" s="0">
+      <c r="D3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G3" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4" t="s" s="0">
+      <c r="A4" t="s">
         <v>0</v>
       </c>
-      <c r="B4" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C4" t="s" s="0">
+      <c r="B4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
         <v>8</v>
       </c>
-      <c r="D4" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E4" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F4" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G4" t="s" s="0">
+      <c r="D4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E4" t="s">
+        <v>3</v>
+      </c>
+      <c r="F4" t="s">
+        <v>4</v>
+      </c>
+      <c r="G4" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A5" t="s" s="0">
+      <c r="A5" t="s">
         <v>0</v>
       </c>
-      <c r="B5" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C5" t="s" s="0">
+      <c r="B5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" t="s">
         <v>10</v>
       </c>
-      <c r="D5" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E5" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F5" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G5" t="s" s="0">
+      <c r="D5" t="s">
+        <v>3</v>
+      </c>
+      <c r="E5" t="s">
+        <v>3</v>
+      </c>
+      <c r="F5" t="s">
+        <v>4</v>
+      </c>
+      <c r="G5" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A6" t="s" s="0">
+      <c r="A6" t="s">
         <v>12</v>
       </c>
-      <c r="B6" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C6" t="s" s="0">
+      <c r="B6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" t="s">
         <v>13</v>
       </c>
-      <c r="D6" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E6" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F6" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G6" t="s" s="0">
+      <c r="D6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E6" t="s">
+        <v>3</v>
+      </c>
+      <c r="F6" t="s">
+        <v>4</v>
+      </c>
+      <c r="G6" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A7" t="s" s="0">
+      <c r="A7" t="s">
         <v>15</v>
       </c>
-      <c r="B7" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C7" t="s" s="0">
+      <c r="B7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" t="s">
         <v>16</v>
       </c>
-      <c r="D7" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E7" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F7" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G7" t="s" s="0">
+      <c r="D7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E7" t="s">
+        <v>3</v>
+      </c>
+      <c r="F7" t="s">
+        <v>4</v>
+      </c>
+      <c r="G7" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A8" t="s" s="0">
+      <c r="A8" t="s">
         <v>18</v>
       </c>
-      <c r="B8" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C8" t="s" s="0">
+      <c r="B8" t="s">
+        <v>1</v>
+      </c>
+      <c r="C8" t="s">
         <v>19</v>
       </c>
-      <c r="D8" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E8" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F8" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G8" t="s" s="0">
+      <c r="D8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E8" t="s">
+        <v>3</v>
+      </c>
+      <c r="F8" t="s">
+        <v>4</v>
+      </c>
+      <c r="G8" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A9" t="s" s="0">
+      <c r="A9" t="s">
         <v>12</v>
       </c>
-      <c r="B9" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C9" t="s" s="0">
+      <c r="B9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
         <v>21</v>
       </c>
-      <c r="D9" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E9" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F9" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G9" t="s" s="0">
+      <c r="D9" t="s">
+        <v>3</v>
+      </c>
+      <c r="E9" t="s">
+        <v>3</v>
+      </c>
+      <c r="F9" t="s">
+        <v>4</v>
+      </c>
+      <c r="G9" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A10" t="s" s="0">
+      <c r="A10" t="s">
         <v>15</v>
       </c>
-      <c r="B10" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C10" t="s" s="0">
+      <c r="B10" t="s">
+        <v>1</v>
+      </c>
+      <c r="C10" t="s">
         <v>23</v>
       </c>
-      <c r="D10" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E10" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F10" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G10" t="s" s="0">
+      <c r="D10" t="s">
+        <v>3</v>
+      </c>
+      <c r="E10" t="s">
+        <v>3</v>
+      </c>
+      <c r="F10" t="s">
+        <v>4</v>
+      </c>
+      <c r="G10" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A11" t="s" s="0">
+      <c r="A11" t="s">
         <v>18</v>
       </c>
-      <c r="B11" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C11" t="s" s="0">
+      <c r="B11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C11" t="s">
         <v>25</v>
       </c>
-      <c r="D11" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E11" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F11" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G11" t="s" s="0">
+      <c r="D11" t="s">
+        <v>3</v>
+      </c>
+      <c r="E11" t="s">
+        <v>3</v>
+      </c>
+      <c r="F11" t="s">
+        <v>4</v>
+      </c>
+      <c r="G11" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A12" t="s" s="0">
+      <c r="A12" t="s">
         <v>12</v>
       </c>
-      <c r="B12" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C12" t="s" s="0">
+      <c r="B12" t="s">
+        <v>1</v>
+      </c>
+      <c r="C12" t="s">
         <v>27</v>
       </c>
-      <c r="D12" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E12" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F12" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G12" t="s" s="0">
+      <c r="D12" t="s">
+        <v>3</v>
+      </c>
+      <c r="E12" t="s">
+        <v>3</v>
+      </c>
+      <c r="F12" t="s">
+        <v>4</v>
+      </c>
+      <c r="G12" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A13" t="s" s="0">
+      <c r="A13" t="s">
         <v>15</v>
       </c>
-      <c r="B13" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C13" t="s" s="0">
+      <c r="B13" t="s">
+        <v>1</v>
+      </c>
+      <c r="C13" t="s">
         <v>29</v>
       </c>
-      <c r="D13" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E13" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F13" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G13" t="s" s="0">
+      <c r="D13" t="s">
+        <v>3</v>
+      </c>
+      <c r="E13" t="s">
+        <v>3</v>
+      </c>
+      <c r="F13" t="s">
+        <v>4</v>
+      </c>
+      <c r="G13" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A14" t="s" s="0">
+      <c r="A14" t="s">
         <v>18</v>
       </c>
-      <c r="B14" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C14" t="s" s="0">
+      <c r="B14" t="s">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
         <v>31</v>
       </c>
-      <c r="D14" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E14" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F14" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G14" t="s" s="0">
+      <c r="D14" t="s">
+        <v>3</v>
+      </c>
+      <c r="E14" t="s">
+        <v>3</v>
+      </c>
+      <c r="F14" t="s">
+        <v>4</v>
+      </c>
+      <c r="G14" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A15" t="s" s="0">
+      <c r="A15" t="s">
         <v>12</v>
       </c>
-      <c r="B15" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C15" t="s" s="0">
+      <c r="B15" t="s">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
         <v>33</v>
       </c>
-      <c r="D15" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E15" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F15" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G15" t="s" s="0">
+      <c r="D15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E15" t="s">
+        <v>3</v>
+      </c>
+      <c r="F15" t="s">
+        <v>4</v>
+      </c>
+      <c r="G15" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A16" t="s" s="0">
+      <c r="A16" t="s">
         <v>15</v>
       </c>
-      <c r="B16" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C16" t="s" s="0">
+      <c r="B16" t="s">
+        <v>1</v>
+      </c>
+      <c r="C16" t="s">
         <v>35</v>
       </c>
-      <c r="D16" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E16" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F16" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G16" t="s" s="0">
+      <c r="D16" t="s">
+        <v>3</v>
+      </c>
+      <c r="E16" t="s">
+        <v>3</v>
+      </c>
+      <c r="F16" t="s">
+        <v>4</v>
+      </c>
+      <c r="G16" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A17" t="s" s="0">
+      <c r="A17" t="s">
         <v>18</v>
       </c>
-      <c r="B17" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C17" t="s" s="0">
+      <c r="B17" t="s">
+        <v>1</v>
+      </c>
+      <c r="C17" t="s">
         <v>37</v>
       </c>
-      <c r="D17" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E17" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F17" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G17" t="s" s="0">
+      <c r="D17" t="s">
+        <v>3</v>
+      </c>
+      <c r="E17" t="s">
+        <v>3</v>
+      </c>
+      <c r="F17" t="s">
+        <v>4</v>
+      </c>
+      <c r="G17" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A18" t="s" s="0">
+      <c r="A18" t="s">
         <v>12</v>
       </c>
-      <c r="B18" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C18" t="s" s="0">
+      <c r="B18" t="s">
+        <v>1</v>
+      </c>
+      <c r="C18" t="s">
         <v>35</v>
       </c>
-      <c r="D18" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E18" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F18" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G18" t="s" s="0">
+      <c r="D18" t="s">
+        <v>3</v>
+      </c>
+      <c r="E18" t="s">
+        <v>3</v>
+      </c>
+      <c r="F18" t="s">
+        <v>4</v>
+      </c>
+      <c r="G18" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A19" t="s" s="0">
+      <c r="A19" t="s">
         <v>15</v>
       </c>
-      <c r="B19" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C19" t="s" s="0">
+      <c r="B19" t="s">
+        <v>1</v>
+      </c>
+      <c r="C19" t="s">
         <v>35</v>
       </c>
-      <c r="D19" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E19" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F19" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G19" t="s" s="0">
+      <c r="D19" t="s">
+        <v>3</v>
+      </c>
+      <c r="E19" t="s">
+        <v>3</v>
+      </c>
+      <c r="F19" t="s">
+        <v>4</v>
+      </c>
+      <c r="G19" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A20" t="s" s="0">
+      <c r="A20" t="s">
         <v>18</v>
       </c>
-      <c r="B20" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C20" t="s" s="0">
+      <c r="B20" t="s">
+        <v>1</v>
+      </c>
+      <c r="C20" t="s">
         <v>35</v>
       </c>
-      <c r="D20" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E20" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F20" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G20" t="s" s="0">
+      <c r="D20" t="s">
+        <v>3</v>
+      </c>
+      <c r="E20" t="s">
+        <v>3</v>
+      </c>
+      <c r="F20" t="s">
+        <v>4</v>
+      </c>
+      <c r="G20" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A21" t="s" s="0">
+      <c r="A21" t="s">
         <v>12</v>
       </c>
-      <c r="B21" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C21" t="s" s="0">
+      <c r="B21" t="s">
+        <v>1</v>
+      </c>
+      <c r="C21" t="s">
         <v>42</v>
       </c>
-      <c r="D21" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E21" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F21" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G21" t="s" s="0">
+      <c r="D21" t="s">
+        <v>3</v>
+      </c>
+      <c r="E21" t="s">
+        <v>3</v>
+      </c>
+      <c r="F21" t="s">
+        <v>4</v>
+      </c>
+      <c r="G21" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A22" t="s" s="0">
+      <c r="A22" t="s">
         <v>15</v>
       </c>
-      <c r="B22" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C22" t="s" s="0">
+      <c r="B22" t="s">
+        <v>1</v>
+      </c>
+      <c r="C22" t="s">
         <v>44</v>
       </c>
-      <c r="D22" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E22" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F22" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G22" t="s" s="0">
+      <c r="D22" t="s">
+        <v>3</v>
+      </c>
+      <c r="E22" t="s">
+        <v>3</v>
+      </c>
+      <c r="F22" t="s">
+        <v>4</v>
+      </c>
+      <c r="G22" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A23" t="s" s="0">
+      <c r="A23" t="s">
         <v>18</v>
       </c>
-      <c r="B23" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C23" t="s" s="0">
+      <c r="B23" t="s">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
         <v>46</v>
       </c>
-      <c r="D23" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E23" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F23" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G23" t="s" s="0">
+      <c r="D23" t="s">
+        <v>3</v>
+      </c>
+      <c r="E23" t="s">
+        <v>3</v>
+      </c>
+      <c r="F23" t="s">
+        <v>4</v>
+      </c>
+      <c r="G23" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A24" t="s" s="0">
+      <c r="A24" t="s">
         <v>12</v>
       </c>
-      <c r="B24" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C24" t="s" s="0">
+      <c r="B24" t="s">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
         <v>48</v>
       </c>
-      <c r="D24" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E24" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F24" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G24" t="s" s="0">
+      <c r="D24" t="s">
+        <v>3</v>
+      </c>
+      <c r="E24" t="s">
+        <v>3</v>
+      </c>
+      <c r="F24" t="s">
+        <v>4</v>
+      </c>
+      <c r="G24" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A25" t="s" s="0">
+      <c r="A25" t="s">
         <v>15</v>
       </c>
-      <c r="B25" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C25" t="s" s="0">
+      <c r="B25" t="s">
+        <v>1</v>
+      </c>
+      <c r="C25" t="s">
         <v>50</v>
       </c>
-      <c r="D25" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E25" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F25" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G25" t="s" s="0">
+      <c r="D25" t="s">
+        <v>3</v>
+      </c>
+      <c r="E25" t="s">
+        <v>3</v>
+      </c>
+      <c r="F25" t="s">
+        <v>4</v>
+      </c>
+      <c r="G25" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A26" t="s" s="0">
+      <c r="A26" t="s">
         <v>18</v>
       </c>
-      <c r="B26" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C26" t="s" s="0">
+      <c r="B26" t="s">
+        <v>1</v>
+      </c>
+      <c r="C26" t="s">
         <v>52</v>
       </c>
-      <c r="D26" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E26" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F26" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G26" t="s" s="0">
+      <c r="D26" t="s">
+        <v>3</v>
+      </c>
+      <c r="E26" t="s">
+        <v>3</v>
+      </c>
+      <c r="F26" t="s">
+        <v>4</v>
+      </c>
+      <c r="G26" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A27" t="s" s="0">
+      <c r="A27" t="s">
         <v>12</v>
       </c>
-      <c r="B27" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C27" t="s" s="0">
+      <c r="B27" t="s">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
         <v>54</v>
       </c>
-      <c r="D27" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E27" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F27" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G27" t="s" s="0">
+      <c r="D27" t="s">
+        <v>3</v>
+      </c>
+      <c r="E27" t="s">
+        <v>3</v>
+      </c>
+      <c r="F27" t="s">
+        <v>4</v>
+      </c>
+      <c r="G27" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A28" t="s" s="0">
+      <c r="A28" t="s">
         <v>15</v>
       </c>
-      <c r="B28" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C28" t="s" s="0">
+      <c r="B28" t="s">
+        <v>1</v>
+      </c>
+      <c r="C28" t="s">
         <v>56</v>
       </c>
-      <c r="D28" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E28" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F28" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G28" t="s" s="0">
+      <c r="D28" t="s">
+        <v>3</v>
+      </c>
+      <c r="E28" t="s">
+        <v>3</v>
+      </c>
+      <c r="F28" t="s">
+        <v>4</v>
+      </c>
+      <c r="G28" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A29" t="s" s="0">
+      <c r="A29" t="s">
         <v>18</v>
       </c>
-      <c r="B29" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C29" t="s" s="0">
+      <c r="B29" t="s">
+        <v>1</v>
+      </c>
+      <c r="C29" t="s">
         <v>58</v>
       </c>
-      <c r="D29" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E29" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F29" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G29" t="s" s="0">
+      <c r="D29" t="s">
+        <v>3</v>
+      </c>
+      <c r="E29" t="s">
+        <v>3</v>
+      </c>
+      <c r="F29" t="s">
+        <v>4</v>
+      </c>
+      <c r="G29" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A30" t="s" s="0">
+      <c r="A30" t="s">
         <v>12</v>
       </c>
-      <c r="B30" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C30" t="s" s="0">
+      <c r="B30" t="s">
+        <v>1</v>
+      </c>
+      <c r="C30" t="s">
         <v>60</v>
       </c>
-      <c r="D30" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E30" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F30" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G30" t="s" s="0">
+      <c r="D30" t="s">
+        <v>3</v>
+      </c>
+      <c r="E30" t="s">
+        <v>3</v>
+      </c>
+      <c r="F30" t="s">
+        <v>4</v>
+      </c>
+      <c r="G30" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A31" t="s" s="0">
+      <c r="A31" t="s">
         <v>15</v>
       </c>
-      <c r="B31" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C31" t="s" s="0">
+      <c r="B31" t="s">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
         <v>62</v>
       </c>
-      <c r="D31" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E31" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F31" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G31" t="s" s="0">
+      <c r="D31" t="s">
+        <v>3</v>
+      </c>
+      <c r="E31" t="s">
+        <v>3</v>
+      </c>
+      <c r="F31" t="s">
+        <v>4</v>
+      </c>
+      <c r="G31" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A32" t="s" s="0">
+      <c r="A32" t="s">
         <v>18</v>
       </c>
-      <c r="B32" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C32" t="s" s="0">
+      <c r="B32" t="s">
+        <v>1</v>
+      </c>
+      <c r="C32" t="s">
         <v>64</v>
       </c>
-      <c r="D32" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E32" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F32" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G32" t="s" s="0">
+      <c r="D32" t="s">
+        <v>3</v>
+      </c>
+      <c r="E32" t="s">
+        <v>3</v>
+      </c>
+      <c r="F32" t="s">
+        <v>4</v>
+      </c>
+      <c r="G32" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A33" t="s" s="0">
+      <c r="A33" t="s">
         <v>12</v>
       </c>
-      <c r="B33" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C33" t="s" s="0">
+      <c r="B33" t="s">
+        <v>1</v>
+      </c>
+      <c r="C33" t="s">
         <v>66</v>
       </c>
-      <c r="D33" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E33" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F33" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G33" t="s" s="0">
+      <c r="D33" t="s">
+        <v>3</v>
+      </c>
+      <c r="E33" t="s">
+        <v>3</v>
+      </c>
+      <c r="F33" t="s">
+        <v>4</v>
+      </c>
+      <c r="G33" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A34" t="s" s="0">
+      <c r="A34" t="s">
         <v>15</v>
       </c>
-      <c r="B34" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C34" t="s" s="0">
+      <c r="B34" t="s">
+        <v>1</v>
+      </c>
+      <c r="C34" t="s">
         <v>68</v>
       </c>
-      <c r="D34" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E34" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F34" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G34" t="s" s="0">
+      <c r="D34" t="s">
+        <v>3</v>
+      </c>
+      <c r="E34" t="s">
+        <v>3</v>
+      </c>
+      <c r="F34" t="s">
+        <v>4</v>
+      </c>
+      <c r="G34" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A35" t="s" s="0">
+      <c r="A35" t="s">
         <v>12</v>
       </c>
-      <c r="B35" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C35" t="s" s="0">
+      <c r="B35" t="s">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
         <v>70</v>
       </c>
-      <c r="D35" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E35" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F35" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G35" t="s" s="0">
+      <c r="D35" t="s">
+        <v>3</v>
+      </c>
+      <c r="E35" t="s">
+        <v>3</v>
+      </c>
+      <c r="F35" t="s">
+        <v>4</v>
+      </c>
+      <c r="G35" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A36" t="s" s="0">
+      <c r="A36" t="s">
         <v>15</v>
       </c>
-      <c r="B36" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C36" t="s" s="0">
+      <c r="B36" t="s">
+        <v>1</v>
+      </c>
+      <c r="C36" t="s">
         <v>72</v>
       </c>
-      <c r="D36" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E36" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F36" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G36" t="s" s="0">
+      <c r="D36" t="s">
+        <v>3</v>
+      </c>
+      <c r="E36" t="s">
+        <v>3</v>
+      </c>
+      <c r="F36" t="s">
+        <v>4</v>
+      </c>
+      <c r="G36" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A37" t="s" s="0">
+      <c r="A37" t="s">
         <v>18</v>
       </c>
-      <c r="B37" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C37" t="s" s="0">
+      <c r="B37" t="s">
+        <v>1</v>
+      </c>
+      <c r="C37" t="s">
         <v>35</v>
       </c>
-      <c r="D37" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E37" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F37" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G37" t="s" s="0">
+      <c r="D37" t="s">
+        <v>3</v>
+      </c>
+      <c r="E37" t="s">
+        <v>3</v>
+      </c>
+      <c r="F37" t="s">
+        <v>4</v>
+      </c>
+      <c r="G37" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A38" t="s" s="0">
+      <c r="A38" t="s">
         <v>12</v>
       </c>
-      <c r="B38" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C38" t="s" s="0">
+      <c r="B38" t="s">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
         <v>75</v>
       </c>
-      <c r="D38" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E38" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F38" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G38" t="s" s="0">
+      <c r="D38" t="s">
+        <v>3</v>
+      </c>
+      <c r="E38" t="s">
+        <v>3</v>
+      </c>
+      <c r="F38" t="s">
+        <v>4</v>
+      </c>
+      <c r="G38" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A39" t="s" s="0">
+      <c r="A39" t="s">
         <v>15</v>
       </c>
-      <c r="B39" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C39" t="s" s="0">
+      <c r="B39" t="s">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
         <v>35</v>
       </c>
-      <c r="D39" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E39" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F39" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G39" t="s" s="0">
+      <c r="D39" t="s">
+        <v>3</v>
+      </c>
+      <c r="E39" t="s">
+        <v>3</v>
+      </c>
+      <c r="F39" t="s">
+        <v>4</v>
+      </c>
+      <c r="G39" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A40" t="s" s="0">
+      <c r="A40" t="s">
         <v>18</v>
       </c>
-      <c r="B40" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C40" t="s" s="0">
+      <c r="B40" t="s">
+        <v>1</v>
+      </c>
+      <c r="C40" t="s">
         <v>78</v>
       </c>
-      <c r="D40" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E40" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F40" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G40" t="s" s="0">
+      <c r="D40" t="s">
+        <v>3</v>
+      </c>
+      <c r="E40" t="s">
+        <v>3</v>
+      </c>
+      <c r="F40" t="s">
+        <v>4</v>
+      </c>
+      <c r="G40" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A41" t="s" s="0">
+      <c r="A41" t="s">
         <v>12</v>
       </c>
-      <c r="B41" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C41" t="s" s="0">
+      <c r="B41" t="s">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
         <v>80</v>
       </c>
-      <c r="D41" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E41" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F41" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G41" t="s" s="0">
+      <c r="D41" t="s">
+        <v>3</v>
+      </c>
+      <c r="E41" t="s">
+        <v>3</v>
+      </c>
+      <c r="F41" t="s">
+        <v>4</v>
+      </c>
+      <c r="G41" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A42" t="s" s="0">
+      <c r="A42" t="s">
         <v>15</v>
       </c>
-      <c r="B42" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C42" t="s" s="0">
+      <c r="B42" t="s">
+        <v>1</v>
+      </c>
+      <c r="C42" t="s">
         <v>82</v>
       </c>
-      <c r="D42" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E42" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F42" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G42" t="s" s="0">
+      <c r="D42" t="s">
+        <v>3</v>
+      </c>
+      <c r="E42" t="s">
+        <v>3</v>
+      </c>
+      <c r="F42" t="s">
+        <v>4</v>
+      </c>
+      <c r="G42" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A43" t="s" s="0">
+      <c r="A43" t="s">
         <v>18</v>
       </c>
-      <c r="B43" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C43" t="s" s="0">
+      <c r="B43" t="s">
+        <v>1</v>
+      </c>
+      <c r="C43" t="s">
         <v>84</v>
       </c>
-      <c r="D43" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E43" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F43" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G43" t="s" s="0">
+      <c r="D43" t="s">
+        <v>3</v>
+      </c>
+      <c r="E43" t="s">
+        <v>3</v>
+      </c>
+      <c r="F43" t="s">
+        <v>4</v>
+      </c>
+      <c r="G43" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A44" t="s" s="0">
+      <c r="A44" t="s">
         <v>12</v>
       </c>
-      <c r="B44" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C44" t="s" s="0">
+      <c r="B44" t="s">
+        <v>1</v>
+      </c>
+      <c r="C44" t="s">
         <v>86</v>
       </c>
-      <c r="D44" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E44" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F44" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G44" t="s" s="0">
+      <c r="D44" t="s">
+        <v>3</v>
+      </c>
+      <c r="E44" t="s">
+        <v>3</v>
+      </c>
+      <c r="F44" t="s">
+        <v>4</v>
+      </c>
+      <c r="G44" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A45" t="s" s="0">
+      <c r="A45" t="s">
         <v>15</v>
       </c>
-      <c r="B45" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C45" t="s" s="0">
+      <c r="B45" t="s">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
         <v>88</v>
       </c>
-      <c r="D45" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E45" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F45" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G45" t="s" s="0">
+      <c r="D45" t="s">
+        <v>3</v>
+      </c>
+      <c r="E45" t="s">
+        <v>3</v>
+      </c>
+      <c r="F45" t="s">
+        <v>4</v>
+      </c>
+      <c r="G45" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A46" t="s" s="0">
+      <c r="A46" t="s">
         <v>18</v>
       </c>
-      <c r="B46" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C46" t="s" s="0">
+      <c r="B46" t="s">
+        <v>1</v>
+      </c>
+      <c r="C46" t="s">
         <v>90</v>
       </c>
-      <c r="D46" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E46" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F46" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G46" t="s" s="0">
+      <c r="D46" t="s">
+        <v>3</v>
+      </c>
+      <c r="E46" t="s">
+        <v>3</v>
+      </c>
+      <c r="F46" t="s">
+        <v>4</v>
+      </c>
+      <c r="G46" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A47" t="s" s="0">
+      <c r="A47" t="s">
         <v>12</v>
       </c>
-      <c r="B47" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C47" t="s" s="0">
+      <c r="B47" t="s">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
         <v>92</v>
       </c>
-      <c r="D47" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E47" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F47" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G47" t="s" s="0">
+      <c r="D47" t="s">
+        <v>3</v>
+      </c>
+      <c r="E47" t="s">
+        <v>3</v>
+      </c>
+      <c r="F47" t="s">
+        <v>4</v>
+      </c>
+      <c r="G47" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A48" t="s" s="0">
+      <c r="A48" t="s">
         <v>15</v>
       </c>
-      <c r="B48" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C48" t="s" s="0">
+      <c r="B48" t="s">
+        <v>1</v>
+      </c>
+      <c r="C48" t="s">
         <v>35</v>
       </c>
-      <c r="D48" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E48" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F48" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G48" t="s" s="0">
+      <c r="D48" t="s">
+        <v>3</v>
+      </c>
+      <c r="E48" t="s">
+        <v>3</v>
+      </c>
+      <c r="F48" t="s">
+        <v>4</v>
+      </c>
+      <c r="G48" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A49" t="s" s="0">
+      <c r="A49" t="s">
         <v>18</v>
       </c>
-      <c r="B49" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C49" t="s" s="0">
+      <c r="B49" t="s">
+        <v>1</v>
+      </c>
+      <c r="C49" t="s">
         <v>35</v>
       </c>
-      <c r="D49" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E49" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F49" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G49" t="s" s="0">
+      <c r="D49" t="s">
+        <v>3</v>
+      </c>
+      <c r="E49" t="s">
+        <v>3</v>
+      </c>
+      <c r="F49" t="s">
+        <v>4</v>
+      </c>
+      <c r="G49" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A50" t="s" s="0">
+      <c r="A50" t="s">
         <v>12</v>
       </c>
-      <c r="B50" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C50" t="s" s="0">
+      <c r="B50" t="s">
+        <v>1</v>
+      </c>
+      <c r="C50" t="s">
         <v>96</v>
       </c>
-      <c r="D50" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E50" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F50" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G50" t="s" s="0">
+      <c r="D50" t="s">
+        <v>3</v>
+      </c>
+      <c r="E50" t="s">
+        <v>3</v>
+      </c>
+      <c r="F50" t="s">
+        <v>4</v>
+      </c>
+      <c r="G50" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A51" t="s" s="0">
+      <c r="A51" t="s">
         <v>15</v>
       </c>
-      <c r="B51" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C51" t="s" s="0">
+      <c r="B51" t="s">
+        <v>1</v>
+      </c>
+      <c r="C51" t="s">
         <v>98</v>
       </c>
-      <c r="D51" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E51" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F51" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G51" t="s" s="0">
+      <c r="D51" t="s">
+        <v>3</v>
+      </c>
+      <c r="E51" t="s">
+        <v>3</v>
+      </c>
+      <c r="F51" t="s">
+        <v>4</v>
+      </c>
+      <c r="G51" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A52" t="s" s="0">
+      <c r="A52" t="s">
         <v>18</v>
       </c>
-      <c r="B52" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C52" t="s" s="0">
+      <c r="B52" t="s">
+        <v>1</v>
+      </c>
+      <c r="C52" t="s">
         <v>100</v>
       </c>
-      <c r="D52" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E52" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F52" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G52" t="s" s="0">
+      <c r="D52" t="s">
+        <v>3</v>
+      </c>
+      <c r="E52" t="s">
+        <v>3</v>
+      </c>
+      <c r="F52" t="s">
+        <v>4</v>
+      </c>
+      <c r="G52" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" t="s" s="0">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
         <v>12</v>
       </c>
-      <c r="B53" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C53" t="s" s="0">
+      <c r="B53" t="s">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>169</v>
+      </c>
+      <c r="D53" t="s">
+        <v>3</v>
+      </c>
+      <c r="E53" t="s">
+        <v>3</v>
+      </c>
+      <c r="F53" t="s">
+        <v>4</v>
+      </c>
+      <c r="G53" t="s">
         <v>170</v>
       </c>
-      <c r="D53" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E53" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F53" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G53" t="s" s="0">
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A54" t="s">
+        <v>15</v>
+      </c>
+      <c r="B54" t="s">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>169</v>
+      </c>
+      <c r="D54" t="s">
+        <v>3</v>
+      </c>
+      <c r="E54" t="s">
+        <v>3</v>
+      </c>
+      <c r="F54" t="s">
+        <v>4</v>
+      </c>
+      <c r="G54" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" t="s" s="0">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
+        <v>18</v>
+      </c>
+      <c r="B55" t="s">
+        <v>1</v>
+      </c>
+      <c r="C55" t="s">
+        <v>169</v>
+      </c>
+      <c r="D55" t="s">
+        <v>3</v>
+      </c>
+      <c r="E55" t="s">
+        <v>3</v>
+      </c>
+      <c r="F55" t="s">
+        <v>4</v>
+      </c>
+      <c r="G55" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
+        <v>12</v>
+      </c>
+      <c r="B56" t="s">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>173</v>
+      </c>
+      <c r="D56" t="s">
+        <v>3</v>
+      </c>
+      <c r="E56" t="s">
+        <v>3</v>
+      </c>
+      <c r="F56" t="s">
+        <v>4</v>
+      </c>
+      <c r="G56" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A57" t="s">
         <v>15</v>
       </c>
-      <c r="B54" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C54" t="s" s="0">
-        <v>170</v>
-      </c>
-      <c r="D54" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E54" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F54" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G54" t="s" s="0">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="s" s="0">
+      <c r="B57" t="s">
+        <v>175</v>
+      </c>
+      <c r="C57" t="s">
+        <v>176</v>
+      </c>
+      <c r="D57" t="s">
+        <v>176</v>
+      </c>
+      <c r="E57" t="s">
+        <v>176</v>
+      </c>
+      <c r="F57" t="s">
+        <v>177</v>
+      </c>
+      <c r="G57" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A58" t="s">
+        <v>15</v>
+      </c>
+      <c r="B58" t="s">
+        <v>175</v>
+      </c>
+      <c r="C58" t="s">
+        <v>176</v>
+      </c>
+      <c r="D58" t="s">
+        <v>176</v>
+      </c>
+      <c r="E58" t="s">
+        <v>176</v>
+      </c>
+      <c r="F58" t="s">
+        <v>177</v>
+      </c>
+      <c r="G58" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A59" t="s">
+        <v>15</v>
+      </c>
+      <c r="B59" t="s">
+        <v>1</v>
+      </c>
+      <c r="C59" t="s">
+        <v>181</v>
+      </c>
+      <c r="D59" t="s">
+        <v>3</v>
+      </c>
+      <c r="E59" t="s">
+        <v>3</v>
+      </c>
+      <c r="F59" t="s">
+        <v>4</v>
+      </c>
+      <c r="G59" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A60" t="s">
         <v>18</v>
       </c>
-      <c r="B55" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C55" t="s" s="0">
-        <v>170</v>
-      </c>
-      <c r="D55" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E55" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F55" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G55" t="s" s="0">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="s" s="0">
+      <c r="B60" t="s">
+        <v>175</v>
+      </c>
+      <c r="C60" t="s">
+        <v>183</v>
+      </c>
+      <c r="D60" t="s">
+        <v>184</v>
+      </c>
+      <c r="E60" t="s">
+        <v>185</v>
+      </c>
+      <c r="F60" t="s">
+        <v>177</v>
+      </c>
+      <c r="G60" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A61" t="s">
+        <v>18</v>
+      </c>
+      <c r="B61" t="s">
+        <v>175</v>
+      </c>
+      <c r="C61" t="s">
+        <v>187</v>
+      </c>
+      <c r="D61" t="s">
+        <v>188</v>
+      </c>
+      <c r="E61" t="s">
+        <v>189</v>
+      </c>
+      <c r="F61" t="s">
+        <v>177</v>
+      </c>
+      <c r="G61" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
+        <v>18</v>
+      </c>
+      <c r="B62" t="s">
+        <v>1</v>
+      </c>
+      <c r="C62" t="s">
+        <v>193</v>
+      </c>
+      <c r="D62" t="s">
+        <v>3</v>
+      </c>
+      <c r="E62" t="s">
+        <v>3</v>
+      </c>
+      <c r="F62" t="s">
+        <v>4</v>
+      </c>
+      <c r="G62" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
         <v>12</v>
       </c>
-      <c r="B56" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C56" t="s" s="0">
-        <v>174</v>
-      </c>
-      <c r="D56" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E56" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F56" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G56" t="s" s="0">
+      <c r="B63" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="s" s="0">
-        <v>15</v>
-      </c>
-      <c r="B57" t="s" s="0">
+      <c r="C63" t="s">
+        <v>195</v>
+      </c>
+      <c r="D63" t="s">
+        <v>196</v>
+      </c>
+      <c r="E63" t="s">
+        <v>197</v>
+      </c>
+      <c r="F63" t="s">
+        <v>177</v>
+      </c>
+      <c r="G63" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A64" t="s">
+        <v>12</v>
+      </c>
+      <c r="B64" t="s">
+        <v>175</v>
+      </c>
+      <c r="C64" t="s">
         <v>176</v>
       </c>
-      <c r="C57" t="s" s="0">
+      <c r="D64" t="s">
+        <v>176</v>
+      </c>
+      <c r="E64" t="s">
+        <v>176</v>
+      </c>
+      <c r="F64" t="s">
         <v>177</v>
       </c>
-      <c r="D57" t="s" s="0">
-        <v>177</v>
-      </c>
-      <c r="E57" t="s" s="0">
-        <v>177</v>
-      </c>
-      <c r="F57" t="s" s="0">
-        <v>178</v>
-      </c>
-      <c r="G57" t="s" s="0">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="s" s="0">
-        <v>15</v>
-      </c>
-      <c r="B58" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="C58" t="s" s="0">
-        <v>177</v>
-      </c>
-      <c r="D58" t="s" s="0">
-        <v>177</v>
-      </c>
-      <c r="E58" t="s" s="0">
-        <v>177</v>
-      </c>
-      <c r="F58" t="s" s="0">
-        <v>178</v>
-      </c>
-      <c r="G58" t="s" s="0">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="s" s="0">
-        <v>15</v>
-      </c>
-      <c r="B59" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C59" t="s" s="0">
-        <v>182</v>
-      </c>
-      <c r="D59" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E59" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F59" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G59" t="s" s="0">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="s" s="0">
-        <v>18</v>
-      </c>
-      <c r="B60" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="C60" t="s" s="0">
-        <v>184</v>
-      </c>
-      <c r="D60" t="s" s="0">
-        <v>185</v>
-      </c>
-      <c r="E60" t="s" s="0">
-        <v>186</v>
-      </c>
-      <c r="F60" t="s" s="0">
-        <v>178</v>
-      </c>
-      <c r="G60" t="s" s="0">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="s" s="0">
-        <v>18</v>
-      </c>
-      <c r="B61" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="C61" t="s" s="0">
-        <v>188</v>
-      </c>
-      <c r="D61" t="s" s="0">
-        <v>189</v>
-      </c>
-      <c r="E61" t="s" s="0">
-        <v>190</v>
-      </c>
-      <c r="F61" t="s" s="0">
-        <v>178</v>
-      </c>
-      <c r="G61" t="s" s="0">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="s" s="0">
-        <v>18</v>
-      </c>
-      <c r="B62" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C62" t="s" s="0">
-        <v>194</v>
-      </c>
-      <c r="D62" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E62" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F62" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G62" t="s" s="0">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="s" s="0">
-        <v>12</v>
-      </c>
-      <c r="B63" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="C63" t="s" s="0">
-        <v>196</v>
-      </c>
-      <c r="D63" t="s" s="0">
-        <v>197</v>
-      </c>
-      <c r="E63" t="s" s="0">
-        <v>198</v>
-      </c>
-      <c r="F63" t="s" s="0">
-        <v>178</v>
-      </c>
-      <c r="G63" t="s" s="0">
+      <c r="G64" t="s">
         <v>199</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="s" s="0">
-        <v>12</v>
-      </c>
-      <c r="B64" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="C64" t="s" s="0">
-        <v>177</v>
-      </c>
-      <c r="D64" t="s" s="0">
-        <v>177</v>
-      </c>
-      <c r="E64" t="s" s="0">
-        <v>177</v>
-      </c>
-      <c r="F64" t="s" s="0">
-        <v>178</v>
-      </c>
-      <c r="G64" t="s" s="0">
-        <v>200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix the course page details locators
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -3,14 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2506400\Desktop\Pooja-Workspace\UdemyAutomation\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FD8CA22-8FA5-41C1-8353-5107B9FB4836}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{822CED62-4E19-42F4-AC57-46851216540B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TestCases" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="614" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="614" uniqueCount="217">
   <si>
     <t>extractCategoryCatalog</t>
   </si>
@@ -924,13 +924,15 @@
   </si>
   <si>
     <t>2026-07-23 09:22:42</t>
+  </si>
+  <si>
+    <t>Advanced</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1308,20 +1310,20 @@
   <dimension ref="A1:U7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="12.0"/>
-    <col min="2" max="2" customWidth="true" width="22.0"/>
-    <col min="3" max="3" customWidth="true" width="14.0"/>
-    <col min="4" max="4" customWidth="true" width="16.0"/>
-    <col min="5" max="6" customWidth="true" width="14.0"/>
-    <col min="7" max="7" customWidth="true" width="22.6328125"/>
-    <col min="8" max="8" customWidth="true" width="14.90625"/>
-    <col min="9" max="14" customWidth="true" hidden="true" width="8.7265625"/>
-    <col min="15" max="15" customWidth="true" width="21.36328125"/>
-    <col min="16" max="16" customWidth="true" width="17.81640625"/>
-    <col min="17" max="17" customWidth="true" width="20.6328125"/>
-    <col min="18" max="18" customWidth="true" width="21.81640625"/>
-    <col min="19" max="20" customWidth="true" width="15.7265625"/>
-    <col min="21" max="21" customWidth="true" width="59.6328125"/>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="6" width="14" customWidth="1"/>
+    <col min="7" max="7" width="22.6328125" customWidth="1"/>
+    <col min="8" max="8" width="14.90625" customWidth="1"/>
+    <col min="9" max="14" width="8.7265625" hidden="1" customWidth="1"/>
+    <col min="15" max="15" width="21.36328125" customWidth="1"/>
+    <col min="16" max="16" width="17.81640625" customWidth="1"/>
+    <col min="17" max="17" width="20.6328125" customWidth="1"/>
+    <col min="18" max="18" width="21.81640625" customWidth="1"/>
+    <col min="19" max="20" width="15.7265625" customWidth="1"/>
+    <col min="21" max="21" width="59.6328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.35">
@@ -1401,29 +1403,29 @@
       <c r="G2" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="H2" t="s" s="0">
+      <c r="H2" t="s">
         <v>139</v>
       </c>
       <c r="I2" s="3"/>
-      <c r="O2" t="s" s="0">
+      <c r="O2" t="s">
         <v>140</v>
       </c>
-      <c r="P2" t="s" s="0">
+      <c r="P2" t="s">
         <v>141</v>
       </c>
       <c r="Q2" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="R2" t="s" s="0">
+      <c r="R2" t="s">
         <v>162</v>
       </c>
-      <c r="S2" t="s" s="0">
+      <c r="S2" t="s">
         <v>163</v>
       </c>
-      <c r="T2" t="s" s="0">
+      <c r="T2" t="s">
         <v>142</v>
       </c>
-      <c r="U2" t="s" s="0">
+      <c r="U2" t="s">
         <v>143</v>
       </c>
     </row>
@@ -1435,7 +1437,7 @@
         <v>114</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>109</v>
+        <v>216</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>110</v>
@@ -1449,29 +1451,29 @@
       <c r="G3" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="H3" t="s" s="0">
+      <c r="H3" t="s">
         <v>148</v>
       </c>
       <c r="I3" s="3"/>
-      <c r="O3" t="s" s="0">
+      <c r="O3" t="s">
         <v>147</v>
       </c>
-      <c r="P3" t="s" s="0">
+      <c r="P3" t="s">
         <v>146</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="R3" t="s" s="0">
+      <c r="R3" t="s">
         <v>164</v>
       </c>
-      <c r="S3" t="s" s="0">
+      <c r="S3" t="s">
         <v>165</v>
       </c>
-      <c r="T3" t="s" s="0">
+      <c r="T3" t="s">
         <v>145</v>
       </c>
-      <c r="U3" t="s" s="0">
+      <c r="U3" t="s">
         <v>144</v>
       </c>
     </row>
@@ -1497,29 +1499,29 @@
       <c r="G4" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="H4" t="s" s="0">
+      <c r="H4" t="s">
         <v>151</v>
       </c>
       <c r="I4" s="3"/>
-      <c r="O4" t="s" s="0">
+      <c r="O4" t="s">
         <v>168</v>
       </c>
-      <c r="P4" t="s" s="0">
+      <c r="P4" t="s">
         <v>152</v>
       </c>
       <c r="Q4" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="R4" t="s" s="0">
+      <c r="R4" t="s">
         <v>166</v>
       </c>
-      <c r="S4" t="s" s="0">
+      <c r="S4" t="s">
         <v>167</v>
       </c>
-      <c r="T4" t="s" s="0">
+      <c r="T4" t="s">
         <v>153</v>
       </c>
-      <c r="U4" t="s" s="0">
+      <c r="U4" t="s">
         <v>154</v>
       </c>
     </row>
@@ -1543,13 +1545,13 @@
   <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="14.08984375"/>
-    <col min="2" max="2" customWidth="true" width="19.453125"/>
-    <col min="3" max="3" customWidth="true" width="19.08984375"/>
-    <col min="4" max="4" customWidth="true" width="8.7265625"/>
-    <col min="5" max="5" customWidth="true" width="17.7265625"/>
-    <col min="6" max="6" customWidth="true" width="14.54296875"/>
-    <col min="7" max="7" customWidth="true" width="15.7265625"/>
+    <col min="1" max="1" width="14.08984375" customWidth="1"/>
+    <col min="2" max="2" width="19.453125" customWidth="1"/>
+    <col min="3" max="3" width="19.08984375" customWidth="1"/>
+    <col min="4" max="4" width="8.7265625" customWidth="1"/>
+    <col min="5" max="5" width="17.7265625" customWidth="1"/>
+    <col min="6" max="6" width="14.54296875" customWidth="1"/>
+    <col min="7" max="7" width="15.7265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
@@ -1576,117 +1578,117 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>15</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s">
         <v>179</v>
       </c>
-      <c r="C2" t="s" s="0">
+      <c r="C2" t="s">
         <v>180</v>
       </c>
-      <c r="D2" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="E2" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="F2" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="G2" t="s" s="0">
+      <c r="D2" t="s">
+        <v>176</v>
+      </c>
+      <c r="E2" t="s">
+        <v>176</v>
+      </c>
+      <c r="F2" t="s">
+        <v>176</v>
+      </c>
+      <c r="G2" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3" t="s" s="0">
+      <c r="A3" t="s">
         <v>18</v>
       </c>
-      <c r="B3" t="s" s="0">
+      <c r="B3" t="s">
         <v>191</v>
       </c>
-      <c r="C3" t="s" s="0">
+      <c r="C3" t="s">
         <v>192</v>
       </c>
-      <c r="D3" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="E3" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="F3" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="G3" t="s" s="0">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s" s="0">
+      <c r="D3" t="s">
+        <v>176</v>
+      </c>
+      <c r="E3" t="s">
+        <v>176</v>
+      </c>
+      <c r="F3" t="s">
+        <v>176</v>
+      </c>
+      <c r="G3" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>12</v>
       </c>
-      <c r="B4" t="s" s="0">
+      <c r="B4" t="s">
         <v>202</v>
       </c>
-      <c r="C4" t="s" s="0">
+      <c r="C4" t="s">
         <v>203</v>
       </c>
-      <c r="D4" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="E4" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="F4" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="G4" t="s" s="0">
+      <c r="D4" t="s">
+        <v>176</v>
+      </c>
+      <c r="E4" t="s">
+        <v>176</v>
+      </c>
+      <c r="F4" t="s">
+        <v>176</v>
+      </c>
+      <c r="G4" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="s" s="0">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>15</v>
       </c>
-      <c r="B5" t="s" s="0">
+      <c r="B5" t="s">
         <v>179</v>
       </c>
-      <c r="C5" t="s" s="0">
+      <c r="C5" t="s">
         <v>180</v>
       </c>
-      <c r="D5" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="E5" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="F5" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="G5" t="s" s="0">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s" s="0">
+      <c r="D5" t="s">
+        <v>176</v>
+      </c>
+      <c r="E5" t="s">
+        <v>176</v>
+      </c>
+      <c r="F5" t="s">
+        <v>176</v>
+      </c>
+      <c r="G5" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
         <v>18</v>
       </c>
-      <c r="B6" t="s" s="0">
+      <c r="B6" t="s">
         <v>191</v>
       </c>
-      <c r="C6" t="s" s="0">
+      <c r="C6" t="s">
         <v>192</v>
       </c>
-      <c r="D6" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="E6" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="F6" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="G6" t="s" s="0">
+      <c r="D6" t="s">
+        <v>176</v>
+      </c>
+      <c r="E6" t="s">
+        <v>176</v>
+      </c>
+      <c r="F6" t="s">
+        <v>176</v>
+      </c>
+      <c r="G6" t="s">
         <v>176</v>
       </c>
     </row>
@@ -1700,12 +1702,12 @@
   <dimension ref="A1:G73"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" customWidth="true" width="12.0"/>
-    <col min="3" max="3" customWidth="true" width="30.0"/>
-    <col min="4" max="4" customWidth="true" width="14.0"/>
-    <col min="5" max="5" customWidth="true" width="12.0"/>
-    <col min="6" max="6" customWidth="true" width="10.0"/>
-    <col min="7" max="7" customWidth="true" width="18.0"/>
+    <col min="1" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="30" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="6" max="6" width="10" customWidth="1"/>
+    <col min="7" max="7" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
@@ -1732,1658 +1734,1658 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C2" t="s" s="0">
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
         <v>2</v>
       </c>
-      <c r="D2" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E2" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F2" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G2" t="s" s="0">
+      <c r="D2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3" t="s" s="0">
+      <c r="A3" t="s">
         <v>0</v>
       </c>
-      <c r="B3" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C3" t="s" s="0">
+      <c r="B3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
         <v>6</v>
       </c>
-      <c r="D3" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E3" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F3" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G3" t="s" s="0">
+      <c r="D3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G3" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4" t="s" s="0">
+      <c r="A4" t="s">
         <v>0</v>
       </c>
-      <c r="B4" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C4" t="s" s="0">
+      <c r="B4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
         <v>8</v>
       </c>
-      <c r="D4" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E4" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F4" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G4" t="s" s="0">
+      <c r="D4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E4" t="s">
+        <v>3</v>
+      </c>
+      <c r="F4" t="s">
+        <v>4</v>
+      </c>
+      <c r="G4" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A5" t="s" s="0">
+      <c r="A5" t="s">
         <v>0</v>
       </c>
-      <c r="B5" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C5" t="s" s="0">
+      <c r="B5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" t="s">
         <v>10</v>
       </c>
-      <c r="D5" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E5" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F5" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G5" t="s" s="0">
+      <c r="D5" t="s">
+        <v>3</v>
+      </c>
+      <c r="E5" t="s">
+        <v>3</v>
+      </c>
+      <c r="F5" t="s">
+        <v>4</v>
+      </c>
+      <c r="G5" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A6" t="s" s="0">
+      <c r="A6" t="s">
         <v>12</v>
       </c>
-      <c r="B6" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C6" t="s" s="0">
+      <c r="B6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" t="s">
         <v>13</v>
       </c>
-      <c r="D6" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E6" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F6" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G6" t="s" s="0">
+      <c r="D6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E6" t="s">
+        <v>3</v>
+      </c>
+      <c r="F6" t="s">
+        <v>4</v>
+      </c>
+      <c r="G6" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A7" t="s" s="0">
+      <c r="A7" t="s">
         <v>15</v>
       </c>
-      <c r="B7" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C7" t="s" s="0">
+      <c r="B7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" t="s">
         <v>16</v>
       </c>
-      <c r="D7" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E7" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F7" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G7" t="s" s="0">
+      <c r="D7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E7" t="s">
+        <v>3</v>
+      </c>
+      <c r="F7" t="s">
+        <v>4</v>
+      </c>
+      <c r="G7" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A8" t="s" s="0">
+      <c r="A8" t="s">
         <v>18</v>
       </c>
-      <c r="B8" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C8" t="s" s="0">
+      <c r="B8" t="s">
+        <v>1</v>
+      </c>
+      <c r="C8" t="s">
         <v>19</v>
       </c>
-      <c r="D8" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E8" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F8" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G8" t="s" s="0">
+      <c r="D8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E8" t="s">
+        <v>3</v>
+      </c>
+      <c r="F8" t="s">
+        <v>4</v>
+      </c>
+      <c r="G8" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A9" t="s" s="0">
+      <c r="A9" t="s">
         <v>12</v>
       </c>
-      <c r="B9" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C9" t="s" s="0">
+      <c r="B9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
         <v>21</v>
       </c>
-      <c r="D9" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E9" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F9" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G9" t="s" s="0">
+      <c r="D9" t="s">
+        <v>3</v>
+      </c>
+      <c r="E9" t="s">
+        <v>3</v>
+      </c>
+      <c r="F9" t="s">
+        <v>4</v>
+      </c>
+      <c r="G9" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A10" t="s" s="0">
+      <c r="A10" t="s">
         <v>15</v>
       </c>
-      <c r="B10" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C10" t="s" s="0">
+      <c r="B10" t="s">
+        <v>1</v>
+      </c>
+      <c r="C10" t="s">
         <v>23</v>
       </c>
-      <c r="D10" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E10" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F10" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G10" t="s" s="0">
+      <c r="D10" t="s">
+        <v>3</v>
+      </c>
+      <c r="E10" t="s">
+        <v>3</v>
+      </c>
+      <c r="F10" t="s">
+        <v>4</v>
+      </c>
+      <c r="G10" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A11" t="s" s="0">
+      <c r="A11" t="s">
         <v>18</v>
       </c>
-      <c r="B11" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C11" t="s" s="0">
+      <c r="B11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C11" t="s">
         <v>25</v>
       </c>
-      <c r="D11" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E11" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F11" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G11" t="s" s="0">
+      <c r="D11" t="s">
+        <v>3</v>
+      </c>
+      <c r="E11" t="s">
+        <v>3</v>
+      </c>
+      <c r="F11" t="s">
+        <v>4</v>
+      </c>
+      <c r="G11" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A12" t="s" s="0">
+      <c r="A12" t="s">
         <v>12</v>
       </c>
-      <c r="B12" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C12" t="s" s="0">
+      <c r="B12" t="s">
+        <v>1</v>
+      </c>
+      <c r="C12" t="s">
         <v>27</v>
       </c>
-      <c r="D12" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E12" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F12" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G12" t="s" s="0">
+      <c r="D12" t="s">
+        <v>3</v>
+      </c>
+      <c r="E12" t="s">
+        <v>3</v>
+      </c>
+      <c r="F12" t="s">
+        <v>4</v>
+      </c>
+      <c r="G12" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A13" t="s" s="0">
+      <c r="A13" t="s">
         <v>15</v>
       </c>
-      <c r="B13" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C13" t="s" s="0">
+      <c r="B13" t="s">
+        <v>1</v>
+      </c>
+      <c r="C13" t="s">
         <v>29</v>
       </c>
-      <c r="D13" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E13" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F13" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G13" t="s" s="0">
+      <c r="D13" t="s">
+        <v>3</v>
+      </c>
+      <c r="E13" t="s">
+        <v>3</v>
+      </c>
+      <c r="F13" t="s">
+        <v>4</v>
+      </c>
+      <c r="G13" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A14" t="s" s="0">
+      <c r="A14" t="s">
         <v>18</v>
       </c>
-      <c r="B14" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C14" t="s" s="0">
+      <c r="B14" t="s">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
         <v>31</v>
       </c>
-      <c r="D14" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E14" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F14" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G14" t="s" s="0">
+      <c r="D14" t="s">
+        <v>3</v>
+      </c>
+      <c r="E14" t="s">
+        <v>3</v>
+      </c>
+      <c r="F14" t="s">
+        <v>4</v>
+      </c>
+      <c r="G14" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A15" t="s" s="0">
+      <c r="A15" t="s">
         <v>12</v>
       </c>
-      <c r="B15" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C15" t="s" s="0">
+      <c r="B15" t="s">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
         <v>33</v>
       </c>
-      <c r="D15" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E15" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F15" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G15" t="s" s="0">
+      <c r="D15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E15" t="s">
+        <v>3</v>
+      </c>
+      <c r="F15" t="s">
+        <v>4</v>
+      </c>
+      <c r="G15" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A16" t="s" s="0">
+      <c r="A16" t="s">
         <v>15</v>
       </c>
-      <c r="B16" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C16" t="s" s="0">
+      <c r="B16" t="s">
+        <v>1</v>
+      </c>
+      <c r="C16" t="s">
         <v>35</v>
       </c>
-      <c r="D16" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E16" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F16" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G16" t="s" s="0">
+      <c r="D16" t="s">
+        <v>3</v>
+      </c>
+      <c r="E16" t="s">
+        <v>3</v>
+      </c>
+      <c r="F16" t="s">
+        <v>4</v>
+      </c>
+      <c r="G16" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A17" t="s" s="0">
+      <c r="A17" t="s">
         <v>18</v>
       </c>
-      <c r="B17" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C17" t="s" s="0">
+      <c r="B17" t="s">
+        <v>1</v>
+      </c>
+      <c r="C17" t="s">
         <v>37</v>
       </c>
-      <c r="D17" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E17" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F17" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G17" t="s" s="0">
+      <c r="D17" t="s">
+        <v>3</v>
+      </c>
+      <c r="E17" t="s">
+        <v>3</v>
+      </c>
+      <c r="F17" t="s">
+        <v>4</v>
+      </c>
+      <c r="G17" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A18" t="s" s="0">
+      <c r="A18" t="s">
         <v>12</v>
       </c>
-      <c r="B18" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C18" t="s" s="0">
+      <c r="B18" t="s">
+        <v>1</v>
+      </c>
+      <c r="C18" t="s">
         <v>35</v>
       </c>
-      <c r="D18" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E18" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F18" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G18" t="s" s="0">
+      <c r="D18" t="s">
+        <v>3</v>
+      </c>
+      <c r="E18" t="s">
+        <v>3</v>
+      </c>
+      <c r="F18" t="s">
+        <v>4</v>
+      </c>
+      <c r="G18" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A19" t="s" s="0">
+      <c r="A19" t="s">
         <v>15</v>
       </c>
-      <c r="B19" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C19" t="s" s="0">
+      <c r="B19" t="s">
+        <v>1</v>
+      </c>
+      <c r="C19" t="s">
         <v>35</v>
       </c>
-      <c r="D19" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E19" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F19" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G19" t="s" s="0">
+      <c r="D19" t="s">
+        <v>3</v>
+      </c>
+      <c r="E19" t="s">
+        <v>3</v>
+      </c>
+      <c r="F19" t="s">
+        <v>4</v>
+      </c>
+      <c r="G19" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A20" t="s" s="0">
+      <c r="A20" t="s">
         <v>18</v>
       </c>
-      <c r="B20" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C20" t="s" s="0">
+      <c r="B20" t="s">
+        <v>1</v>
+      </c>
+      <c r="C20" t="s">
         <v>35</v>
       </c>
-      <c r="D20" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E20" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F20" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G20" t="s" s="0">
+      <c r="D20" t="s">
+        <v>3</v>
+      </c>
+      <c r="E20" t="s">
+        <v>3</v>
+      </c>
+      <c r="F20" t="s">
+        <v>4</v>
+      </c>
+      <c r="G20" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A21" t="s" s="0">
+      <c r="A21" t="s">
         <v>12</v>
       </c>
-      <c r="B21" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C21" t="s" s="0">
+      <c r="B21" t="s">
+        <v>1</v>
+      </c>
+      <c r="C21" t="s">
         <v>42</v>
       </c>
-      <c r="D21" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E21" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F21" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G21" t="s" s="0">
+      <c r="D21" t="s">
+        <v>3</v>
+      </c>
+      <c r="E21" t="s">
+        <v>3</v>
+      </c>
+      <c r="F21" t="s">
+        <v>4</v>
+      </c>
+      <c r="G21" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A22" t="s" s="0">
+      <c r="A22" t="s">
         <v>15</v>
       </c>
-      <c r="B22" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C22" t="s" s="0">
+      <c r="B22" t="s">
+        <v>1</v>
+      </c>
+      <c r="C22" t="s">
         <v>44</v>
       </c>
-      <c r="D22" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E22" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F22" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G22" t="s" s="0">
+      <c r="D22" t="s">
+        <v>3</v>
+      </c>
+      <c r="E22" t="s">
+        <v>3</v>
+      </c>
+      <c r="F22" t="s">
+        <v>4</v>
+      </c>
+      <c r="G22" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A23" t="s" s="0">
+      <c r="A23" t="s">
         <v>18</v>
       </c>
-      <c r="B23" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C23" t="s" s="0">
+      <c r="B23" t="s">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
         <v>46</v>
       </c>
-      <c r="D23" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E23" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F23" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G23" t="s" s="0">
+      <c r="D23" t="s">
+        <v>3</v>
+      </c>
+      <c r="E23" t="s">
+        <v>3</v>
+      </c>
+      <c r="F23" t="s">
+        <v>4</v>
+      </c>
+      <c r="G23" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A24" t="s" s="0">
+      <c r="A24" t="s">
         <v>12</v>
       </c>
-      <c r="B24" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C24" t="s" s="0">
+      <c r="B24" t="s">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
         <v>48</v>
       </c>
-      <c r="D24" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E24" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F24" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G24" t="s" s="0">
+      <c r="D24" t="s">
+        <v>3</v>
+      </c>
+      <c r="E24" t="s">
+        <v>3</v>
+      </c>
+      <c r="F24" t="s">
+        <v>4</v>
+      </c>
+      <c r="G24" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A25" t="s" s="0">
+      <c r="A25" t="s">
         <v>15</v>
       </c>
-      <c r="B25" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C25" t="s" s="0">
+      <c r="B25" t="s">
+        <v>1</v>
+      </c>
+      <c r="C25" t="s">
         <v>50</v>
       </c>
-      <c r="D25" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E25" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F25" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G25" t="s" s="0">
+      <c r="D25" t="s">
+        <v>3</v>
+      </c>
+      <c r="E25" t="s">
+        <v>3</v>
+      </c>
+      <c r="F25" t="s">
+        <v>4</v>
+      </c>
+      <c r="G25" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A26" t="s" s="0">
+      <c r="A26" t="s">
         <v>18</v>
       </c>
-      <c r="B26" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C26" t="s" s="0">
+      <c r="B26" t="s">
+        <v>1</v>
+      </c>
+      <c r="C26" t="s">
         <v>52</v>
       </c>
-      <c r="D26" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E26" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F26" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G26" t="s" s="0">
+      <c r="D26" t="s">
+        <v>3</v>
+      </c>
+      <c r="E26" t="s">
+        <v>3</v>
+      </c>
+      <c r="F26" t="s">
+        <v>4</v>
+      </c>
+      <c r="G26" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A27" t="s" s="0">
+      <c r="A27" t="s">
         <v>12</v>
       </c>
-      <c r="B27" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C27" t="s" s="0">
+      <c r="B27" t="s">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
         <v>54</v>
       </c>
-      <c r="D27" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E27" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F27" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G27" t="s" s="0">
+      <c r="D27" t="s">
+        <v>3</v>
+      </c>
+      <c r="E27" t="s">
+        <v>3</v>
+      </c>
+      <c r="F27" t="s">
+        <v>4</v>
+      </c>
+      <c r="G27" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A28" t="s" s="0">
+      <c r="A28" t="s">
         <v>15</v>
       </c>
-      <c r="B28" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C28" t="s" s="0">
+      <c r="B28" t="s">
+        <v>1</v>
+      </c>
+      <c r="C28" t="s">
         <v>56</v>
       </c>
-      <c r="D28" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E28" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F28" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G28" t="s" s="0">
+      <c r="D28" t="s">
+        <v>3</v>
+      </c>
+      <c r="E28" t="s">
+        <v>3</v>
+      </c>
+      <c r="F28" t="s">
+        <v>4</v>
+      </c>
+      <c r="G28" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A29" t="s" s="0">
+      <c r="A29" t="s">
         <v>18</v>
       </c>
-      <c r="B29" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C29" t="s" s="0">
+      <c r="B29" t="s">
+        <v>1</v>
+      </c>
+      <c r="C29" t="s">
         <v>58</v>
       </c>
-      <c r="D29" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E29" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F29" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G29" t="s" s="0">
+      <c r="D29" t="s">
+        <v>3</v>
+      </c>
+      <c r="E29" t="s">
+        <v>3</v>
+      </c>
+      <c r="F29" t="s">
+        <v>4</v>
+      </c>
+      <c r="G29" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A30" t="s" s="0">
+      <c r="A30" t="s">
         <v>12</v>
       </c>
-      <c r="B30" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C30" t="s" s="0">
+      <c r="B30" t="s">
+        <v>1</v>
+      </c>
+      <c r="C30" t="s">
         <v>60</v>
       </c>
-      <c r="D30" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E30" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F30" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G30" t="s" s="0">
+      <c r="D30" t="s">
+        <v>3</v>
+      </c>
+      <c r="E30" t="s">
+        <v>3</v>
+      </c>
+      <c r="F30" t="s">
+        <v>4</v>
+      </c>
+      <c r="G30" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A31" t="s" s="0">
+      <c r="A31" t="s">
         <v>15</v>
       </c>
-      <c r="B31" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C31" t="s" s="0">
+      <c r="B31" t="s">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
         <v>62</v>
       </c>
-      <c r="D31" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E31" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F31" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G31" t="s" s="0">
+      <c r="D31" t="s">
+        <v>3</v>
+      </c>
+      <c r="E31" t="s">
+        <v>3</v>
+      </c>
+      <c r="F31" t="s">
+        <v>4</v>
+      </c>
+      <c r="G31" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A32" t="s" s="0">
+      <c r="A32" t="s">
         <v>18</v>
       </c>
-      <c r="B32" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C32" t="s" s="0">
+      <c r="B32" t="s">
+        <v>1</v>
+      </c>
+      <c r="C32" t="s">
         <v>64</v>
       </c>
-      <c r="D32" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E32" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F32" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G32" t="s" s="0">
+      <c r="D32" t="s">
+        <v>3</v>
+      </c>
+      <c r="E32" t="s">
+        <v>3</v>
+      </c>
+      <c r="F32" t="s">
+        <v>4</v>
+      </c>
+      <c r="G32" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A33" t="s" s="0">
+      <c r="A33" t="s">
         <v>12</v>
       </c>
-      <c r="B33" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C33" t="s" s="0">
+      <c r="B33" t="s">
+        <v>1</v>
+      </c>
+      <c r="C33" t="s">
         <v>66</v>
       </c>
-      <c r="D33" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E33" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F33" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G33" t="s" s="0">
+      <c r="D33" t="s">
+        <v>3</v>
+      </c>
+      <c r="E33" t="s">
+        <v>3</v>
+      </c>
+      <c r="F33" t="s">
+        <v>4</v>
+      </c>
+      <c r="G33" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A34" t="s" s="0">
+      <c r="A34" t="s">
         <v>15</v>
       </c>
-      <c r="B34" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C34" t="s" s="0">
+      <c r="B34" t="s">
+        <v>1</v>
+      </c>
+      <c r="C34" t="s">
         <v>68</v>
       </c>
-      <c r="D34" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E34" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F34" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G34" t="s" s="0">
+      <c r="D34" t="s">
+        <v>3</v>
+      </c>
+      <c r="E34" t="s">
+        <v>3</v>
+      </c>
+      <c r="F34" t="s">
+        <v>4</v>
+      </c>
+      <c r="G34" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A35" t="s" s="0">
+      <c r="A35" t="s">
         <v>12</v>
       </c>
-      <c r="B35" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C35" t="s" s="0">
+      <c r="B35" t="s">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
         <v>70</v>
       </c>
-      <c r="D35" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E35" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F35" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G35" t="s" s="0">
+      <c r="D35" t="s">
+        <v>3</v>
+      </c>
+      <c r="E35" t="s">
+        <v>3</v>
+      </c>
+      <c r="F35" t="s">
+        <v>4</v>
+      </c>
+      <c r="G35" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A36" t="s" s="0">
+      <c r="A36" t="s">
         <v>15</v>
       </c>
-      <c r="B36" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C36" t="s" s="0">
+      <c r="B36" t="s">
+        <v>1</v>
+      </c>
+      <c r="C36" t="s">
         <v>72</v>
       </c>
-      <c r="D36" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E36" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F36" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G36" t="s" s="0">
+      <c r="D36" t="s">
+        <v>3</v>
+      </c>
+      <c r="E36" t="s">
+        <v>3</v>
+      </c>
+      <c r="F36" t="s">
+        <v>4</v>
+      </c>
+      <c r="G36" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A37" t="s" s="0">
+      <c r="A37" t="s">
         <v>18</v>
       </c>
-      <c r="B37" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C37" t="s" s="0">
+      <c r="B37" t="s">
+        <v>1</v>
+      </c>
+      <c r="C37" t="s">
         <v>35</v>
       </c>
-      <c r="D37" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E37" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F37" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G37" t="s" s="0">
+      <c r="D37" t="s">
+        <v>3</v>
+      </c>
+      <c r="E37" t="s">
+        <v>3</v>
+      </c>
+      <c r="F37" t="s">
+        <v>4</v>
+      </c>
+      <c r="G37" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A38" t="s" s="0">
+      <c r="A38" t="s">
         <v>12</v>
       </c>
-      <c r="B38" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C38" t="s" s="0">
+      <c r="B38" t="s">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
         <v>75</v>
       </c>
-      <c r="D38" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E38" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F38" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G38" t="s" s="0">
+      <c r="D38" t="s">
+        <v>3</v>
+      </c>
+      <c r="E38" t="s">
+        <v>3</v>
+      </c>
+      <c r="F38" t="s">
+        <v>4</v>
+      </c>
+      <c r="G38" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A39" t="s" s="0">
+      <c r="A39" t="s">
         <v>15</v>
       </c>
-      <c r="B39" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C39" t="s" s="0">
+      <c r="B39" t="s">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
         <v>35</v>
       </c>
-      <c r="D39" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E39" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F39" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G39" t="s" s="0">
+      <c r="D39" t="s">
+        <v>3</v>
+      </c>
+      <c r="E39" t="s">
+        <v>3</v>
+      </c>
+      <c r="F39" t="s">
+        <v>4</v>
+      </c>
+      <c r="G39" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A40" t="s" s="0">
+      <c r="A40" t="s">
         <v>18</v>
       </c>
-      <c r="B40" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C40" t="s" s="0">
+      <c r="B40" t="s">
+        <v>1</v>
+      </c>
+      <c r="C40" t="s">
         <v>78</v>
       </c>
-      <c r="D40" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E40" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F40" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G40" t="s" s="0">
+      <c r="D40" t="s">
+        <v>3</v>
+      </c>
+      <c r="E40" t="s">
+        <v>3</v>
+      </c>
+      <c r="F40" t="s">
+        <v>4</v>
+      </c>
+      <c r="G40" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A41" t="s" s="0">
+      <c r="A41" t="s">
         <v>12</v>
       </c>
-      <c r="B41" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C41" t="s" s="0">
+      <c r="B41" t="s">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
         <v>80</v>
       </c>
-      <c r="D41" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E41" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F41" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G41" t="s" s="0">
+      <c r="D41" t="s">
+        <v>3</v>
+      </c>
+      <c r="E41" t="s">
+        <v>3</v>
+      </c>
+      <c r="F41" t="s">
+        <v>4</v>
+      </c>
+      <c r="G41" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A42" t="s" s="0">
+      <c r="A42" t="s">
         <v>15</v>
       </c>
-      <c r="B42" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C42" t="s" s="0">
+      <c r="B42" t="s">
+        <v>1</v>
+      </c>
+      <c r="C42" t="s">
         <v>82</v>
       </c>
-      <c r="D42" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E42" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F42" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G42" t="s" s="0">
+      <c r="D42" t="s">
+        <v>3</v>
+      </c>
+      <c r="E42" t="s">
+        <v>3</v>
+      </c>
+      <c r="F42" t="s">
+        <v>4</v>
+      </c>
+      <c r="G42" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A43" t="s" s="0">
+      <c r="A43" t="s">
         <v>18</v>
       </c>
-      <c r="B43" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C43" t="s" s="0">
+      <c r="B43" t="s">
+        <v>1</v>
+      </c>
+      <c r="C43" t="s">
         <v>84</v>
       </c>
-      <c r="D43" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E43" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F43" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G43" t="s" s="0">
+      <c r="D43" t="s">
+        <v>3</v>
+      </c>
+      <c r="E43" t="s">
+        <v>3</v>
+      </c>
+      <c r="F43" t="s">
+        <v>4</v>
+      </c>
+      <c r="G43" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A44" t="s" s="0">
+      <c r="A44" t="s">
         <v>12</v>
       </c>
-      <c r="B44" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C44" t="s" s="0">
+      <c r="B44" t="s">
+        <v>1</v>
+      </c>
+      <c r="C44" t="s">
         <v>86</v>
       </c>
-      <c r="D44" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E44" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F44" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G44" t="s" s="0">
+      <c r="D44" t="s">
+        <v>3</v>
+      </c>
+      <c r="E44" t="s">
+        <v>3</v>
+      </c>
+      <c r="F44" t="s">
+        <v>4</v>
+      </c>
+      <c r="G44" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A45" t="s" s="0">
+      <c r="A45" t="s">
         <v>15</v>
       </c>
-      <c r="B45" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C45" t="s" s="0">
+      <c r="B45" t="s">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
         <v>88</v>
       </c>
-      <c r="D45" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E45" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F45" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G45" t="s" s="0">
+      <c r="D45" t="s">
+        <v>3</v>
+      </c>
+      <c r="E45" t="s">
+        <v>3</v>
+      </c>
+      <c r="F45" t="s">
+        <v>4</v>
+      </c>
+      <c r="G45" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A46" t="s" s="0">
+      <c r="A46" t="s">
         <v>18</v>
       </c>
-      <c r="B46" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C46" t="s" s="0">
+      <c r="B46" t="s">
+        <v>1</v>
+      </c>
+      <c r="C46" t="s">
         <v>90</v>
       </c>
-      <c r="D46" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E46" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F46" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G46" t="s" s="0">
+      <c r="D46" t="s">
+        <v>3</v>
+      </c>
+      <c r="E46" t="s">
+        <v>3</v>
+      </c>
+      <c r="F46" t="s">
+        <v>4</v>
+      </c>
+      <c r="G46" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A47" t="s" s="0">
+      <c r="A47" t="s">
         <v>12</v>
       </c>
-      <c r="B47" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C47" t="s" s="0">
+      <c r="B47" t="s">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
         <v>92</v>
       </c>
-      <c r="D47" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E47" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F47" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G47" t="s" s="0">
+      <c r="D47" t="s">
+        <v>3</v>
+      </c>
+      <c r="E47" t="s">
+        <v>3</v>
+      </c>
+      <c r="F47" t="s">
+        <v>4</v>
+      </c>
+      <c r="G47" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A48" t="s" s="0">
+      <c r="A48" t="s">
         <v>15</v>
       </c>
-      <c r="B48" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C48" t="s" s="0">
+      <c r="B48" t="s">
+        <v>1</v>
+      </c>
+      <c r="C48" t="s">
         <v>35</v>
       </c>
-      <c r="D48" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E48" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F48" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G48" t="s" s="0">
+      <c r="D48" t="s">
+        <v>3</v>
+      </c>
+      <c r="E48" t="s">
+        <v>3</v>
+      </c>
+      <c r="F48" t="s">
+        <v>4</v>
+      </c>
+      <c r="G48" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A49" t="s" s="0">
+      <c r="A49" t="s">
         <v>18</v>
       </c>
-      <c r="B49" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C49" t="s" s="0">
+      <c r="B49" t="s">
+        <v>1</v>
+      </c>
+      <c r="C49" t="s">
         <v>35</v>
       </c>
-      <c r="D49" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E49" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F49" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G49" t="s" s="0">
+      <c r="D49" t="s">
+        <v>3</v>
+      </c>
+      <c r="E49" t="s">
+        <v>3</v>
+      </c>
+      <c r="F49" t="s">
+        <v>4</v>
+      </c>
+      <c r="G49" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A50" t="s" s="0">
+      <c r="A50" t="s">
         <v>12</v>
       </c>
-      <c r="B50" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C50" t="s" s="0">
+      <c r="B50" t="s">
+        <v>1</v>
+      </c>
+      <c r="C50" t="s">
         <v>96</v>
       </c>
-      <c r="D50" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E50" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F50" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G50" t="s" s="0">
+      <c r="D50" t="s">
+        <v>3</v>
+      </c>
+      <c r="E50" t="s">
+        <v>3</v>
+      </c>
+      <c r="F50" t="s">
+        <v>4</v>
+      </c>
+      <c r="G50" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A51" t="s" s="0">
+      <c r="A51" t="s">
         <v>15</v>
       </c>
-      <c r="B51" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C51" t="s" s="0">
+      <c r="B51" t="s">
+        <v>1</v>
+      </c>
+      <c r="C51" t="s">
         <v>98</v>
       </c>
-      <c r="D51" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E51" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F51" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G51" t="s" s="0">
+      <c r="D51" t="s">
+        <v>3</v>
+      </c>
+      <c r="E51" t="s">
+        <v>3</v>
+      </c>
+      <c r="F51" t="s">
+        <v>4</v>
+      </c>
+      <c r="G51" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A52" t="s" s="0">
+      <c r="A52" t="s">
         <v>18</v>
       </c>
-      <c r="B52" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C52" t="s" s="0">
+      <c r="B52" t="s">
+        <v>1</v>
+      </c>
+      <c r="C52" t="s">
         <v>100</v>
       </c>
-      <c r="D52" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E52" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F52" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G52" t="s" s="0">
+      <c r="D52" t="s">
+        <v>3</v>
+      </c>
+      <c r="E52" t="s">
+        <v>3</v>
+      </c>
+      <c r="F52" t="s">
+        <v>4</v>
+      </c>
+      <c r="G52" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A53" t="s" s="0">
+      <c r="A53" t="s">
         <v>12</v>
       </c>
-      <c r="B53" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C53" t="s" s="0">
+      <c r="B53" t="s">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
         <v>169</v>
       </c>
-      <c r="D53" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E53" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F53" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G53" t="s" s="0">
+      <c r="D53" t="s">
+        <v>3</v>
+      </c>
+      <c r="E53" t="s">
+        <v>3</v>
+      </c>
+      <c r="F53" t="s">
+        <v>4</v>
+      </c>
+      <c r="G53" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A54" t="s" s="0">
+      <c r="A54" t="s">
         <v>15</v>
       </c>
-      <c r="B54" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C54" t="s" s="0">
+      <c r="B54" t="s">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
         <v>169</v>
       </c>
-      <c r="D54" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E54" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F54" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G54" t="s" s="0">
+      <c r="D54" t="s">
+        <v>3</v>
+      </c>
+      <c r="E54" t="s">
+        <v>3</v>
+      </c>
+      <c r="F54" t="s">
+        <v>4</v>
+      </c>
+      <c r="G54" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A55" t="s" s="0">
+      <c r="A55" t="s">
         <v>18</v>
       </c>
-      <c r="B55" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C55" t="s" s="0">
+      <c r="B55" t="s">
+        <v>1</v>
+      </c>
+      <c r="C55" t="s">
         <v>169</v>
       </c>
-      <c r="D55" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E55" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F55" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G55" t="s" s="0">
+      <c r="D55" t="s">
+        <v>3</v>
+      </c>
+      <c r="E55" t="s">
+        <v>3</v>
+      </c>
+      <c r="F55" t="s">
+        <v>4</v>
+      </c>
+      <c r="G55" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A56" t="s" s="0">
+      <c r="A56" t="s">
         <v>12</v>
       </c>
-      <c r="B56" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C56" t="s" s="0">
+      <c r="B56" t="s">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
         <v>173</v>
       </c>
-      <c r="D56" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E56" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F56" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G56" t="s" s="0">
+      <c r="D56" t="s">
+        <v>3</v>
+      </c>
+      <c r="E56" t="s">
+        <v>3</v>
+      </c>
+      <c r="F56" t="s">
+        <v>4</v>
+      </c>
+      <c r="G56" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A57" t="s" s="0">
+      <c r="A57" t="s">
         <v>15</v>
       </c>
-      <c r="B57" t="s" s="0">
+      <c r="B57" t="s">
         <v>175</v>
       </c>
-      <c r="C57" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="D57" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="E57" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="F57" t="s" s="0">
+      <c r="C57" t="s">
+        <v>176</v>
+      </c>
+      <c r="D57" t="s">
+        <v>176</v>
+      </c>
+      <c r="E57" t="s">
+        <v>176</v>
+      </c>
+      <c r="F57" t="s">
         <v>177</v>
       </c>
-      <c r="G57" t="s" s="0">
+      <c r="G57" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A58" t="s" s="0">
+      <c r="A58" t="s">
         <v>15</v>
       </c>
-      <c r="B58" t="s" s="0">
+      <c r="B58" t="s">
         <v>175</v>
       </c>
-      <c r="C58" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="D58" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="E58" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="F58" t="s" s="0">
+      <c r="C58" t="s">
+        <v>176</v>
+      </c>
+      <c r="D58" t="s">
+        <v>176</v>
+      </c>
+      <c r="E58" t="s">
+        <v>176</v>
+      </c>
+      <c r="F58" t="s">
         <v>177</v>
       </c>
-      <c r="G58" t="s" s="0">
+      <c r="G58" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A59" t="s" s="0">
+      <c r="A59" t="s">
         <v>15</v>
       </c>
-      <c r="B59" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C59" t="s" s="0">
+      <c r="B59" t="s">
+        <v>1</v>
+      </c>
+      <c r="C59" t="s">
         <v>181</v>
       </c>
-      <c r="D59" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E59" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F59" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G59" t="s" s="0">
+      <c r="D59" t="s">
+        <v>3</v>
+      </c>
+      <c r="E59" t="s">
+        <v>3</v>
+      </c>
+      <c r="F59" t="s">
+        <v>4</v>
+      </c>
+      <c r="G59" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A60" t="s" s="0">
+      <c r="A60" t="s">
         <v>18</v>
       </c>
-      <c r="B60" t="s" s="0">
+      <c r="B60" t="s">
         <v>175</v>
       </c>
-      <c r="C60" t="s" s="0">
+      <c r="C60" t="s">
         <v>183</v>
       </c>
-      <c r="D60" t="s" s="0">
+      <c r="D60" t="s">
         <v>184</v>
       </c>
-      <c r="E60" t="s" s="0">
+      <c r="E60" t="s">
         <v>185</v>
       </c>
-      <c r="F60" t="s" s="0">
+      <c r="F60" t="s">
         <v>177</v>
       </c>
-      <c r="G60" t="s" s="0">
+      <c r="G60" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A61" t="s" s="0">
+      <c r="A61" t="s">
         <v>18</v>
       </c>
-      <c r="B61" t="s" s="0">
+      <c r="B61" t="s">
         <v>175</v>
       </c>
-      <c r="C61" t="s" s="0">
+      <c r="C61" t="s">
         <v>187</v>
       </c>
-      <c r="D61" t="s" s="0">
+      <c r="D61" t="s">
         <v>188</v>
       </c>
-      <c r="E61" t="s" s="0">
+      <c r="E61" t="s">
         <v>189</v>
       </c>
-      <c r="F61" t="s" s="0">
+      <c r="F61" t="s">
         <v>177</v>
       </c>
-      <c r="G61" t="s" s="0">
+      <c r="G61" t="s">
         <v>190</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A62" t="s" s="0">
+      <c r="A62" t="s">
         <v>18</v>
       </c>
-      <c r="B62" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C62" t="s" s="0">
+      <c r="B62" t="s">
+        <v>1</v>
+      </c>
+      <c r="C62" t="s">
         <v>193</v>
       </c>
-      <c r="D62" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E62" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F62" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G62" t="s" s="0">
+      <c r="D62" t="s">
+        <v>3</v>
+      </c>
+      <c r="E62" t="s">
+        <v>3</v>
+      </c>
+      <c r="F62" t="s">
+        <v>4</v>
+      </c>
+      <c r="G62" t="s">
         <v>194</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A63" t="s" s="0">
+      <c r="A63" t="s">
         <v>12</v>
       </c>
-      <c r="B63" t="s" s="0">
+      <c r="B63" t="s">
         <v>175</v>
       </c>
-      <c r="C63" t="s" s="0">
+      <c r="C63" t="s">
         <v>195</v>
       </c>
-      <c r="D63" t="s" s="0">
+      <c r="D63" t="s">
         <v>196</v>
       </c>
-      <c r="E63" t="s" s="0">
+      <c r="E63" t="s">
         <v>197</v>
       </c>
-      <c r="F63" t="s" s="0">
+      <c r="F63" t="s">
         <v>177</v>
       </c>
-      <c r="G63" t="s" s="0">
+      <c r="G63" t="s">
         <v>198</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A64" t="s" s="0">
+      <c r="A64" t="s">
         <v>12</v>
       </c>
-      <c r="B64" t="s" s="0">
+      <c r="B64" t="s">
         <v>175</v>
       </c>
-      <c r="C64" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="D64" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="E64" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="F64" t="s" s="0">
+      <c r="C64" t="s">
+        <v>176</v>
+      </c>
+      <c r="D64" t="s">
+        <v>176</v>
+      </c>
+      <c r="E64" t="s">
+        <v>176</v>
+      </c>
+      <c r="F64" t="s">
         <v>177</v>
       </c>
-      <c r="G64" t="s" s="0">
+      <c r="G64" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" t="s" s="0">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A65" t="s">
         <v>12</v>
       </c>
-      <c r="B65" t="s" s="0">
+      <c r="B65" t="s">
         <v>175</v>
       </c>
-      <c r="C65" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="D65" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="E65" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="F65" t="s" s="0">
+      <c r="C65" t="s">
+        <v>176</v>
+      </c>
+      <c r="D65" t="s">
+        <v>176</v>
+      </c>
+      <c r="E65" t="s">
+        <v>176</v>
+      </c>
+      <c r="F65" t="s">
         <v>177</v>
       </c>
-      <c r="G65" t="s" s="0">
+      <c r="G65" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" t="s" s="0">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A66" t="s">
         <v>12</v>
       </c>
-      <c r="B66" t="s" s="0">
+      <c r="B66" t="s">
         <v>175</v>
       </c>
-      <c r="C66" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="D66" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="E66" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="F66" t="s" s="0">
+      <c r="C66" t="s">
+        <v>176</v>
+      </c>
+      <c r="D66" t="s">
+        <v>176</v>
+      </c>
+      <c r="E66" t="s">
+        <v>176</v>
+      </c>
+      <c r="F66" t="s">
         <v>177</v>
       </c>
-      <c r="G66" t="s" s="0">
+      <c r="G66" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" t="s" s="0">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A67" t="s">
         <v>12</v>
       </c>
-      <c r="B67" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C67" t="s" s="0">
+      <c r="B67" t="s">
+        <v>1</v>
+      </c>
+      <c r="C67" t="s">
         <v>205</v>
       </c>
-      <c r="D67" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E67" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F67" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G67" t="s" s="0">
+      <c r="D67" t="s">
+        <v>3</v>
+      </c>
+      <c r="E67" t="s">
+        <v>3</v>
+      </c>
+      <c r="F67" t="s">
+        <v>4</v>
+      </c>
+      <c r="G67" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" t="s" s="0">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A68" t="s">
         <v>15</v>
       </c>
-      <c r="B68" t="s" s="0">
+      <c r="B68" t="s">
         <v>175</v>
       </c>
-      <c r="C68" t="s" s="0">
+      <c r="C68" t="s">
         <v>179</v>
       </c>
-      <c r="D68" t="s" s="0">
+      <c r="D68" t="s">
         <v>184</v>
       </c>
-      <c r="E68" t="s" s="0">
+      <c r="E68" t="s">
         <v>207</v>
       </c>
-      <c r="F68" t="s" s="0">
+      <c r="F68" t="s">
         <v>177</v>
       </c>
-      <c r="G68" t="s" s="0">
+      <c r="G68" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" t="s" s="0">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
         <v>15</v>
       </c>
-      <c r="B69" t="s" s="0">
+      <c r="B69" t="s">
         <v>175</v>
       </c>
-      <c r="C69" t="s" s="0">
+      <c r="C69" t="s">
         <v>209</v>
       </c>
-      <c r="D69" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="E69" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="F69" t="s" s="0">
+      <c r="D69" t="s">
+        <v>176</v>
+      </c>
+      <c r="E69" t="s">
+        <v>176</v>
+      </c>
+      <c r="F69" t="s">
         <v>177</v>
       </c>
-      <c r="G69" t="s" s="0">
+      <c r="G69" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" t="s" s="0">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A70" t="s">
         <v>15</v>
       </c>
-      <c r="B70" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C70" t="s" s="0">
+      <c r="B70" t="s">
+        <v>1</v>
+      </c>
+      <c r="C70" t="s">
         <v>211</v>
       </c>
-      <c r="D70" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E70" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F70" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G70" t="s" s="0">
+      <c r="D70" t="s">
+        <v>3</v>
+      </c>
+      <c r="E70" t="s">
+        <v>3</v>
+      </c>
+      <c r="F70" t="s">
+        <v>4</v>
+      </c>
+      <c r="G70" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" t="s" s="0">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
         <v>18</v>
       </c>
-      <c r="B71" t="s" s="0">
+      <c r="B71" t="s">
         <v>175</v>
       </c>
-      <c r="C71" t="s" s="0">
+      <c r="C71" t="s">
         <v>183</v>
       </c>
-      <c r="D71" t="s" s="0">
+      <c r="D71" t="s">
         <v>184</v>
       </c>
-      <c r="E71" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="F71" t="s" s="0">
+      <c r="E71" t="s">
+        <v>176</v>
+      </c>
+      <c r="F71" t="s">
         <v>177</v>
       </c>
-      <c r="G71" t="s" s="0">
+      <c r="G71" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" t="s" s="0">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A72" t="s">
         <v>18</v>
       </c>
-      <c r="B72" t="s" s="0">
+      <c r="B72" t="s">
         <v>175</v>
       </c>
-      <c r="C72" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="D72" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="E72" t="s" s="0">
-        <v>176</v>
-      </c>
-      <c r="F72" t="s" s="0">
+      <c r="C72" t="s">
+        <v>176</v>
+      </c>
+      <c r="D72" t="s">
+        <v>176</v>
+      </c>
+      <c r="E72" t="s">
+        <v>176</v>
+      </c>
+      <c r="F72" t="s">
         <v>177</v>
       </c>
-      <c r="G72" t="s" s="0">
+      <c r="G72" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" t="s" s="0">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A73" t="s">
         <v>18</v>
       </c>
-      <c r="B73" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C73" t="s" s="0">
+      <c r="B73" t="s">
+        <v>1</v>
+      </c>
+      <c r="C73" t="s">
         <v>214</v>
       </c>
-      <c r="D73" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E73" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F73" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G73" t="s" s="0">
+      <c r="D73" t="s">
+        <v>3</v>
+      </c>
+      <c r="E73" t="s">
+        <v>3</v>
+      </c>
+      <c r="F73" t="s">
+        <v>4</v>
+      </c>
+      <c r="G73" t="s">
         <v>215</v>
       </c>
     </row>

</xml_diff>

<commit_message>
improve the test flow and added email correction after validation
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -3,7 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{C75C1DEA-AFBD-454E-B052-333317D71C01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent>
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2506400\Desktop\Pooja-Workspace\UdemyAutomation\src\test\resources\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{271A3CA7-F507-442F-9EAC-EEBCCF029BD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -13,7 +18,6 @@
     <sheet name="TestResults" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="C1:N35"/>
   <extLst>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="2"/>
@@ -23,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="662" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="834" uniqueCount="269">
   <si>
     <t>extractCategoryCatalog</t>
   </si>
@@ -574,12 +578,6 @@
   </si>
   <si>
     <t>Aisha</t>
-  </si>
-  <si>
-    <t>Khan</t>
-  </si>
-  <si>
-    <t>aisha.khan@@test.com</t>
   </si>
   <si>
     <t>python programming</t>
@@ -1009,6 +1007,107 @@
   </si>
   <si>
     <t>Expected validation message expected [false] but found [true]</t>
+  </si>
+  <si>
+    <t>Khanna</t>
+  </si>
+  <si>
+    <t>aisha.khanna@@test.com</t>
+  </si>
+  <si>
+    <t>CorrectWorkEmail</t>
+  </si>
+  <si>
+    <t>2026-07-23 16:48:36</t>
+  </si>
+  <si>
+    <t>2026-07-23 16:48:37</t>
+  </si>
+  <si>
+    <t>Advanced Diploma in Python Programming for the Novice to Expert</t>
+  </si>
+  <si>
+    <t>Python is a popular programming language because it is fast, versatile and easy to understand. This free online Python course will hone your passion for programming by taking you through the fundamentals and more advanced features of Python. You will learn exactly how Python programming works, the different applications that Python can work for such as software development and mathematical computations and which areas you can apply them in.</t>
+  </si>
+  <si>
+    <t>15-20
+Avg. Hours</t>
+  </si>
+  <si>
+    <t>36,027</t>
+  </si>
+  <si>
+    <t>Juan Galvan</t>
+  </si>
+  <si>
+    <t>EMAIL_VALIDATION</t>
+  </si>
+  <si>
+    <t>2026-07-23 16:49:27</t>
+  </si>
+  <si>
+    <t>Expected condition failed: waiting for element to be clickable: By.xpath: //button[@class="apply-now-button alison-button alison-button-lg alison-accent-hover w-full mdc-button mdc-button--unelevated mat-mdc-unelevated-button mat-primary mat-mdc-button-base"] (tried for 20 second(s) with 500 milliseconds interval)
+Build info: version: '4.21.0', revision: '79ed462ef4'
+System info: os.name: 'Windows 11', os.arch: 'amd64', os.version: '10.0', java.version: '21.0.10'
+Driver info: org.openqa.selenium.chrome.ChromeDriver
+Capabilities {acceptInsecureCerts: false, browserName: chrome, browserVersion: 150.0.7871.47, chrome: {chromedriverVersion: 150.0.7871.124 (9261fd0a595..., userDataDir: C:\Users\2506400\AppData\Lo...}, fedcm:accounts: true, goog:chromeOptions: {debuggerAddress: localhost:64817}, goog:processID: 16376, networkConnectionEnabled: false, pageLoadStrategy: normal, platformName: windows, proxy: Proxy(), se:cdp: ws://localhost:64817/devtoo..., se:cdpVersion: 150.0.7871.47, setWindowRect: true, strictFileInteractability: false, timeouts: {implicit: 0, pageLoad: 300000, script: 30000}, unhandledPromptBehavior: dismiss and notify, webauthn:extension:credBlob: true, webauthn:extension:largeBlob: true, webauthn:extension:minPinLength: true, webauthn:extension:prf: true, webauthn:virtualAuthenticators: true}
+Session ID: 33007764a451675714d6e801e9cda5c7</t>
+  </si>
+  <si>
+    <t>2026-07-23 16:50:01</t>
+  </si>
+  <si>
+    <t>Expected condition failed: waiting for element to be clickable: By.xpath: //div[@data-url-var='level']//label[contains(translate(normalize-space(.),'ABCDEFGHIJKLMNOPQRSTUVWXYZ','abcdefghijklmnopqrstuvwxyz'),'intermediate')] (tried for 20 second(s) with 500 milliseconds interval)
+Build info: version: '4.21.0', revision: '79ed462ef4'
+System info: os.name: 'Windows 11', os.arch: 'amd64', os.version: '10.0', java.version: '21.0.10'
+Driver info: org.openqa.selenium.chrome.ChromeDriver
+Capabilities {acceptInsecureCerts: false, browserName: chrome, browserVersion: 150.0.7871.47, chrome: {chromedriverVersion: 150.0.7871.124 (9261fd0a595..., userDataDir: C:\Users\2506400\AppData\Lo...}, fedcm:accounts: true, goog:chromeOptions: {debuggerAddress: localhost:52919}, goog:processID: 28980, networkConnectionEnabled: false, pageLoadStrategy: normal, platformName: windows, proxy: Proxy(), se:cdp: ws://localhost:52919/devtoo..., se:cdpVersion: 150.0.7871.47, setWindowRect: true, strictFileInteractability: false, timeouts: {implicit: 0, pageLoad: 300000, script: 30000}, unhandledPromptBehavior: dismiss and notify, webauthn:extension:credBlob: true, webauthn:extension:largeBlob: true, webauthn:extension:minPinLength: true, webauthn:extension:prf: true, webauthn:virtualAuthenticators: true}
+Session ID: fbab62ba6dbae2f6748cdf7563778a43</t>
+  </si>
+  <si>
+    <t>2026-07-23 16:50:57</t>
+  </si>
+  <si>
+    <t>rohanverma@globallearning.com</t>
+  </si>
+  <si>
+    <t>neha.sharma@acmecorp.com</t>
+  </si>
+  <si>
+    <t>aisha.khanna@techsolutions.com</t>
+  </si>
+  <si>
+    <t>2026-07-23 16:55:20</t>
+  </si>
+  <si>
+    <t>2026-07-23 16:55:21</t>
+  </si>
+  <si>
+    <t>2026-07-23 16:56:07</t>
+  </si>
+  <si>
+    <t>2026-07-23 16:56:41</t>
+  </si>
+  <si>
+    <t>2026-07-23 16:57:19</t>
+  </si>
+  <si>
+    <t>2026-07-23 16:58:03</t>
+  </si>
+  <si>
+    <t>2026-07-23 16:58:39</t>
+  </si>
+  <si>
+    <t>2026-07-23 16:58:40</t>
+  </si>
+  <si>
+    <t>2026-07-23 16:59:20</t>
+  </si>
+  <si>
+    <t>2026-07-23 17:00:03</t>
+  </si>
+  <si>
+    <t>2026-07-23 17:00:42</t>
   </si>
 </sst>
 </file>
@@ -1016,7 +1115,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="0"/>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1046,6 +1145,14 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -1070,17 +1177,20 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1381,7 +1491,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:P4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="12.0"/>
@@ -1397,14 +1507,15 @@
     <col min="12" max="12" customWidth="true" width="21.81640625"/>
     <col min="13" max="14" customWidth="true" width="15.7265625"/>
     <col min="15" max="15" customWidth="true" width="59.6328125"/>
+    <col min="16" max="16" customWidth="true" width="30.1796875"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>102</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>103</v>
@@ -1422,31 +1533,34 @@
         <v>107</v>
       </c>
       <c r="H1" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="J1" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="L1" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>154</v>
-      </c>
       <c r="N1" s="3" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
+        <v>135</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>12</v>
       </c>
@@ -1463,145 +1577,159 @@
         <v>111</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>112</v>
+        <v>239</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>113</v>
+        <v>240</v>
       </c>
       <c r="H2" t="s" s="0">
+        <v>136</v>
+      </c>
+      <c r="I2" t="s" s="0">
+        <v>137</v>
+      </c>
+      <c r="J2" t="s" s="0">
         <v>138</v>
       </c>
-      <c r="I2" t="s" s="0">
+      <c r="K2" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="L2" t="s" s="0">
+        <v>201</v>
+      </c>
+      <c r="M2" t="s" s="0">
+        <v>206</v>
+      </c>
+      <c r="N2" t="s" s="0">
         <v>139</v>
       </c>
-      <c r="J2" t="s" s="0">
+      <c r="O2" t="s" s="0">
         <v>140</v>
       </c>
-      <c r="K2" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="L2" t="s" s="0">
-        <v>203</v>
-      </c>
-      <c r="M2" t="s" s="0">
-        <v>208</v>
-      </c>
-      <c r="N2" t="s" s="0">
-        <v>141</v>
-      </c>
-      <c r="O2" t="s" s="0">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P2" s="5" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>15</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>110</v>
       </c>
       <c r="E3" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="F3" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>117</v>
-      </c>
       <c r="H3" t="s" s="0">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="I3" t="s" s="0">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="J3" t="s" s="0">
+        <v>197</v>
+      </c>
+      <c r="K3" s="4" t="s">
         <v>199</v>
       </c>
-      <c r="K3" s="4" t="s">
-        <v>201</v>
-      </c>
       <c r="L3" t="s" s="0">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="M3" t="s" s="0">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="N3" t="s" s="0">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="O3" t="s" s="0">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
+        <v>141</v>
+      </c>
+      <c r="P3" s="5" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>18</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>110</v>
       </c>
       <c r="E4" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="F4" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>122</v>
-      </c>
       <c r="H4" t="s" s="0">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="I4" t="s" s="0">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="L4" t="s" s="0">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="M4" t="s" s="0">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="N4" t="s" s="0">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="O4" t="s" s="0">
-        <v>147</v>
+        <v>145</v>
+      </c>
+      <c r="P4" s="5" t="s">
+        <v>256</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="P2" r:id="rId1" xr:uid="{F112C923-A704-4492-AC2E-CEC6BAD5B2F2}"/>
+    <hyperlink ref="P3" r:id="rId2" xr:uid="{D1DE8963-5799-4847-B581-587BEC77A4BB}"/>
+    <hyperlink ref="P4" r:id="rId3" xr:uid="{7562E8E1-0730-4C56-B6EC-13E719D11723}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId4"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88BFA3FA-6A41-46D8-9F46-57C4912E9286}">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="14.08984375"/>
-    <col min="2" max="2" customWidth="true" width="19.453125"/>
-    <col min="3" max="3" customWidth="true" width="19.08984375"/>
-    <col min="4" max="4" customWidth="true" width="8.7265625"/>
+    <col min="2" max="2" customWidth="true" width="37.54296875"/>
+    <col min="3" max="3" customWidth="true" width="30.453125"/>
+    <col min="4" max="4" customWidth="true" width="18.7265625"/>
     <col min="5" max="5" customWidth="true" width="17.7265625"/>
     <col min="6" max="6" customWidth="true" width="14.54296875"/>
     <col min="7" max="7" customWidth="true" width="15.7265625"/>
@@ -1612,68 +1740,160 @@
         <v>102</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="2">
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s" s="0">
         <v>12</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="C2" t="s" s="0">
+        <v>214</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>215</v>
+      </c>
+      <c r="E2" t="s" s="0">
         <v>216</v>
       </c>
-      <c r="D2" t="s" s="0">
+      <c r="F2" t="s" s="0">
         <v>217</v>
       </c>
-      <c r="E2" t="s" s="0">
+      <c r="G2" t="s" s="0">
         <v>218</v>
       </c>
-      <c r="F2" t="s" s="0">
-        <v>219</v>
-      </c>
-      <c r="G2" t="s" s="0">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="3">
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s" s="0">
         <v>18</v>
       </c>
       <c r="B3" t="s" s="0">
+        <v>231</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>232</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>215</v>
+      </c>
+      <c r="E3" t="s" s="0">
         <v>233</v>
       </c>
-      <c r="C3" t="s" s="0">
+      <c r="F3" t="s" s="0">
         <v>234</v>
       </c>
-      <c r="D3" t="s" s="0">
+      <c r="G3" t="s" s="0">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>244</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>245</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>246</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>247</v>
+      </c>
+      <c r="F4" t="s" s="0">
         <v>217</v>
       </c>
-      <c r="E3" t="s" s="0">
+      <c r="G4" t="s" s="0">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>210</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>214</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>215</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>216</v>
+      </c>
+      <c r="F5" t="s" s="0">
+        <v>217</v>
+      </c>
+      <c r="G5" t="s" s="0">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>244</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>245</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>246</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>247</v>
+      </c>
+      <c r="F6" t="s" s="0">
+        <v>217</v>
+      </c>
+      <c r="G6" t="s" s="0">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>231</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>232</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>215</v>
+      </c>
+      <c r="E7" t="s" s="0">
+        <v>233</v>
+      </c>
+      <c r="F7" t="s" s="0">
+        <v>234</v>
+      </c>
+      <c r="G7" t="s" s="0">
         <v>235</v>
-      </c>
-      <c r="F3" t="s" s="0">
-        <v>236</v>
-      </c>
-      <c r="G3" t="s" s="0">
-        <v>237</v>
       </c>
     </row>
   </sheetData>
@@ -1683,7 +1903,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G83"/>
+  <dimension ref="A1:G103"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" customWidth="true" width="12.0"/>
@@ -1699,22 +1919,22 @@
         <v>102</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>126</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
@@ -2898,7 +3118,7 @@
         <v>1</v>
       </c>
       <c r="C53" t="s" s="0">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="D53" t="s" s="0">
         <v>3</v>
@@ -2910,7 +3130,7 @@
         <v>4</v>
       </c>
       <c r="G53" t="s" s="0">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.35">
@@ -2921,19 +3141,19 @@
         <v>1</v>
       </c>
       <c r="C54" t="s" s="0">
+        <v>154</v>
+      </c>
+      <c r="D54" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E54" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F54" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="G54" t="s" s="0">
         <v>156</v>
-      </c>
-      <c r="D54" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E54" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="F54" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G54" t="s" s="0">
-        <v>158</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.35">
@@ -2944,7 +3164,7 @@
         <v>1</v>
       </c>
       <c r="C55" t="s" s="0">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="D55" t="s" s="0">
         <v>3</v>
@@ -2956,7 +3176,7 @@
         <v>4</v>
       </c>
       <c r="G55" t="s" s="0">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.35">
@@ -2967,7 +3187,7 @@
         <v>1</v>
       </c>
       <c r="C56" t="s" s="0">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="D56" t="s" s="0">
         <v>3</v>
@@ -2979,7 +3199,7 @@
         <v>4</v>
       </c>
       <c r="G56" t="s" s="0">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.35">
@@ -2987,22 +3207,22 @@
         <v>15</v>
       </c>
       <c r="B57" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C57" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="D57" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="E57" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="F57" t="s" s="0">
         <v>162</v>
       </c>
-      <c r="C57" t="s" s="0">
+      <c r="G57" t="s" s="0">
         <v>163</v>
-      </c>
-      <c r="D57" t="s" s="0">
-        <v>163</v>
-      </c>
-      <c r="E57" t="s" s="0">
-        <v>163</v>
-      </c>
-      <c r="F57" t="s" s="0">
-        <v>164</v>
-      </c>
-      <c r="G57" t="s" s="0">
-        <v>165</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.35">
@@ -3010,22 +3230,22 @@
         <v>15</v>
       </c>
       <c r="B58" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C58" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="D58" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="E58" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="F58" t="s" s="0">
         <v>162</v>
       </c>
-      <c r="C58" t="s" s="0">
+      <c r="G58" t="s" s="0">
         <v>163</v>
-      </c>
-      <c r="D58" t="s" s="0">
-        <v>163</v>
-      </c>
-      <c r="E58" t="s" s="0">
-        <v>163</v>
-      </c>
-      <c r="F58" t="s" s="0">
-        <v>164</v>
-      </c>
-      <c r="G58" t="s" s="0">
-        <v>165</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.35">
@@ -3036,7 +3256,7 @@
         <v>1</v>
       </c>
       <c r="C59" t="s" s="0">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="D59" t="s" s="0">
         <v>3</v>
@@ -3048,7 +3268,7 @@
         <v>4</v>
       </c>
       <c r="G59" t="s" s="0">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.35">
@@ -3056,22 +3276,22 @@
         <v>18</v>
       </c>
       <c r="B60" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C60" t="s" s="0">
+        <v>167</v>
+      </c>
+      <c r="D60" t="s" s="0">
+        <v>168</v>
+      </c>
+      <c r="E60" t="s" s="0">
+        <v>169</v>
+      </c>
+      <c r="F60" t="s" s="0">
         <v>162</v>
       </c>
-      <c r="C60" t="s" s="0">
-        <v>169</v>
-      </c>
-      <c r="D60" t="s" s="0">
+      <c r="G60" t="s" s="0">
         <v>170</v>
-      </c>
-      <c r="E60" t="s" s="0">
-        <v>171</v>
-      </c>
-      <c r="F60" t="s" s="0">
-        <v>164</v>
-      </c>
-      <c r="G60" t="s" s="0">
-        <v>172</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.35">
@@ -3079,22 +3299,22 @@
         <v>18</v>
       </c>
       <c r="B61" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C61" t="s" s="0">
+        <v>171</v>
+      </c>
+      <c r="D61" t="s" s="0">
+        <v>172</v>
+      </c>
+      <c r="E61" t="s" s="0">
+        <v>173</v>
+      </c>
+      <c r="F61" t="s" s="0">
         <v>162</v>
       </c>
-      <c r="C61" t="s" s="0">
-        <v>173</v>
-      </c>
-      <c r="D61" t="s" s="0">
+      <c r="G61" t="s" s="0">
         <v>174</v>
-      </c>
-      <c r="E61" t="s" s="0">
-        <v>175</v>
-      </c>
-      <c r="F61" t="s" s="0">
-        <v>164</v>
-      </c>
-      <c r="G61" t="s" s="0">
-        <v>176</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.35">
@@ -3105,7 +3325,7 @@
         <v>1</v>
       </c>
       <c r="C62" t="s" s="0">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D62" t="s" s="0">
         <v>3</v>
@@ -3117,7 +3337,7 @@
         <v>4</v>
       </c>
       <c r="G62" t="s" s="0">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.35">
@@ -3125,22 +3345,22 @@
         <v>12</v>
       </c>
       <c r="B63" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C63" t="s" s="0">
+        <v>177</v>
+      </c>
+      <c r="D63" t="s" s="0">
+        <v>178</v>
+      </c>
+      <c r="E63" t="s" s="0">
+        <v>179</v>
+      </c>
+      <c r="F63" t="s" s="0">
         <v>162</v>
       </c>
-      <c r="C63" t="s" s="0">
-        <v>179</v>
-      </c>
-      <c r="D63" t="s" s="0">
+      <c r="G63" t="s" s="0">
         <v>180</v>
-      </c>
-      <c r="E63" t="s" s="0">
-        <v>181</v>
-      </c>
-      <c r="F63" t="s" s="0">
-        <v>164</v>
-      </c>
-      <c r="G63" t="s" s="0">
-        <v>182</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.35">
@@ -3148,22 +3368,22 @@
         <v>12</v>
       </c>
       <c r="B64" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C64" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="D64" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="E64" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="F64" t="s" s="0">
         <v>162</v>
       </c>
-      <c r="C64" t="s" s="0">
-        <v>163</v>
-      </c>
-      <c r="D64" t="s" s="0">
-        <v>163</v>
-      </c>
-      <c r="E64" t="s" s="0">
-        <v>163</v>
-      </c>
-      <c r="F64" t="s" s="0">
-        <v>164</v>
-      </c>
       <c r="G64" t="s" s="0">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.35">
@@ -3171,22 +3391,22 @@
         <v>12</v>
       </c>
       <c r="B65" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C65" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="D65" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="E65" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="F65" t="s" s="0">
         <v>162</v>
       </c>
-      <c r="C65" t="s" s="0">
-        <v>163</v>
-      </c>
-      <c r="D65" t="s" s="0">
-        <v>163</v>
-      </c>
-      <c r="E65" t="s" s="0">
-        <v>163</v>
-      </c>
-      <c r="F65" t="s" s="0">
-        <v>164</v>
-      </c>
       <c r="G65" t="s" s="0">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.35">
@@ -3194,22 +3414,22 @@
         <v>12</v>
       </c>
       <c r="B66" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C66" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="D66" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="E66" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="F66" t="s" s="0">
         <v>162</v>
       </c>
-      <c r="C66" t="s" s="0">
-        <v>163</v>
-      </c>
-      <c r="D66" t="s" s="0">
-        <v>163</v>
-      </c>
-      <c r="E66" t="s" s="0">
-        <v>163</v>
-      </c>
-      <c r="F66" t="s" s="0">
-        <v>164</v>
-      </c>
       <c r="G66" t="s" s="0">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.35">
@@ -3220,7 +3440,7 @@
         <v>1</v>
       </c>
       <c r="C67" t="s" s="0">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="D67" t="s" s="0">
         <v>3</v>
@@ -3232,7 +3452,7 @@
         <v>4</v>
       </c>
       <c r="G67" t="s" s="0">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.35">
@@ -3240,22 +3460,22 @@
         <v>15</v>
       </c>
       <c r="B68" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C68" t="s" s="0">
+        <v>164</v>
+      </c>
+      <c r="D68" t="s" s="0">
+        <v>168</v>
+      </c>
+      <c r="E68" t="s" s="0">
+        <v>186</v>
+      </c>
+      <c r="F68" t="s" s="0">
         <v>162</v>
       </c>
-      <c r="C68" t="s" s="0">
-        <v>166</v>
-      </c>
-      <c r="D68" t="s" s="0">
-        <v>170</v>
-      </c>
-      <c r="E68" t="s" s="0">
-        <v>188</v>
-      </c>
-      <c r="F68" t="s" s="0">
-        <v>164</v>
-      </c>
       <c r="G68" t="s" s="0">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.35">
@@ -3263,22 +3483,22 @@
         <v>15</v>
       </c>
       <c r="B69" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C69" t="s" s="0">
+        <v>188</v>
+      </c>
+      <c r="D69" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="E69" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="F69" t="s" s="0">
         <v>162</v>
       </c>
-      <c r="C69" t="s" s="0">
-        <v>190</v>
-      </c>
-      <c r="D69" t="s" s="0">
-        <v>163</v>
-      </c>
-      <c r="E69" t="s" s="0">
-        <v>163</v>
-      </c>
-      <c r="F69" t="s" s="0">
-        <v>164</v>
-      </c>
       <c r="G69" t="s" s="0">
-        <v>191</v>
+        <v>189</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.35">
@@ -3289,7 +3509,7 @@
         <v>1</v>
       </c>
       <c r="C70" t="s" s="0">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="D70" t="s" s="0">
         <v>3</v>
@@ -3301,7 +3521,7 @@
         <v>4</v>
       </c>
       <c r="G70" t="s" s="0">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.35">
@@ -3309,22 +3529,22 @@
         <v>18</v>
       </c>
       <c r="B71" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C71" t="s" s="0">
+        <v>167</v>
+      </c>
+      <c r="D71" t="s" s="0">
+        <v>168</v>
+      </c>
+      <c r="E71" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="F71" t="s" s="0">
         <v>162</v>
       </c>
-      <c r="C71" t="s" s="0">
-        <v>169</v>
-      </c>
-      <c r="D71" t="s" s="0">
-        <v>170</v>
-      </c>
-      <c r="E71" t="s" s="0">
-        <v>163</v>
-      </c>
-      <c r="F71" t="s" s="0">
-        <v>164</v>
-      </c>
       <c r="G71" t="s" s="0">
-        <v>194</v>
+        <v>192</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.35">
@@ -3332,22 +3552,22 @@
         <v>18</v>
       </c>
       <c r="B72" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C72" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="D72" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="E72" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="F72" t="s" s="0">
         <v>162</v>
       </c>
-      <c r="C72" t="s" s="0">
-        <v>163</v>
-      </c>
-      <c r="D72" t="s" s="0">
-        <v>163</v>
-      </c>
-      <c r="E72" t="s" s="0">
-        <v>163</v>
-      </c>
-      <c r="F72" t="s" s="0">
-        <v>164</v>
-      </c>
       <c r="G72" t="s" s="0">
-        <v>194</v>
+        <v>192</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.35">
@@ -3358,7 +3578,7 @@
         <v>1</v>
       </c>
       <c r="C73" t="s" s="0">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="D73" t="s" s="0">
         <v>3</v>
@@ -3370,56 +3590,56 @@
         <v>4</v>
       </c>
       <c r="G73" t="s" s="0">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="74">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A74" t="s" s="0">
         <v>12</v>
       </c>
       <c r="B74" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C74" t="s" s="0">
+        <v>177</v>
+      </c>
+      <c r="D74" t="s" s="0">
+        <v>178</v>
+      </c>
+      <c r="E74" t="s" s="0">
+        <v>208</v>
+      </c>
+      <c r="F74" t="s" s="0">
         <v>162</v>
       </c>
-      <c r="C74" t="s" s="0">
-        <v>179</v>
-      </c>
-      <c r="D74" t="s" s="0">
-        <v>180</v>
-      </c>
-      <c r="E74" t="s" s="0">
-        <v>210</v>
-      </c>
-      <c r="F74" t="s" s="0">
-        <v>164</v>
-      </c>
       <c r="G74" t="s" s="0">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="75">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A75" t="s" s="0">
         <v>12</v>
       </c>
       <c r="B75" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C75" t="s" s="0">
+        <v>210</v>
+      </c>
+      <c r="D75" t="s" s="0">
+        <v>211</v>
+      </c>
+      <c r="E75" t="s" s="0">
+        <v>212</v>
+      </c>
+      <c r="F75" t="s" s="0">
         <v>162</v>
       </c>
-      <c r="C75" t="s" s="0">
-        <v>212</v>
-      </c>
-      <c r="D75" t="s" s="0">
+      <c r="G75" t="s" s="0">
         <v>213</v>
       </c>
-      <c r="E75" t="s" s="0">
-        <v>214</v>
-      </c>
-      <c r="F75" t="s" s="0">
-        <v>164</v>
-      </c>
-      <c r="G75" t="s" s="0">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="76">
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A76" t="s" s="0">
         <v>12</v>
       </c>
@@ -3427,7 +3647,7 @@
         <v>1</v>
       </c>
       <c r="C76" t="s" s="0">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="D76" t="s" s="0">
         <v>3</v>
@@ -3439,56 +3659,56 @@
         <v>4</v>
       </c>
       <c r="G76" t="s" s="0">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="77">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A77" t="s" s="0">
         <v>15</v>
       </c>
       <c r="B77" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C77" t="s" s="0">
+        <v>164</v>
+      </c>
+      <c r="D77" t="s" s="0">
+        <v>168</v>
+      </c>
+      <c r="E77" t="s" s="0">
+        <v>221</v>
+      </c>
+      <c r="F77" t="s" s="0">
         <v>162</v>
       </c>
-      <c r="C77" t="s" s="0">
-        <v>166</v>
-      </c>
-      <c r="D77" t="s" s="0">
-        <v>170</v>
-      </c>
-      <c r="E77" t="s" s="0">
-        <v>223</v>
-      </c>
-      <c r="F77" t="s" s="0">
-        <v>164</v>
-      </c>
       <c r="G77" t="s" s="0">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="78">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A78" t="s" s="0">
         <v>15</v>
       </c>
       <c r="B78" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C78" t="s" s="0">
+        <v>188</v>
+      </c>
+      <c r="D78" t="s" s="0">
+        <v>223</v>
+      </c>
+      <c r="E78" t="s" s="0">
+        <v>224</v>
+      </c>
+      <c r="F78" t="s" s="0">
         <v>162</v>
       </c>
-      <c r="C78" t="s" s="0">
-        <v>190</v>
-      </c>
-      <c r="D78" t="s" s="0">
+      <c r="G78" t="s" s="0">
         <v>225</v>
       </c>
-      <c r="E78" t="s" s="0">
-        <v>226</v>
-      </c>
-      <c r="F78" t="s" s="0">
-        <v>164</v>
-      </c>
-      <c r="G78" t="s" s="0">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="79">
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A79" t="s" s="0">
         <v>15</v>
       </c>
@@ -3496,7 +3716,7 @@
         <v>1</v>
       </c>
       <c r="C79" t="s" s="0">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="D79" t="s" s="0">
         <v>3</v>
@@ -3508,61 +3728,61 @@
         <v>4</v>
       </c>
       <c r="G79" t="s" s="0">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="80">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A80" t="s" s="0">
         <v>18</v>
       </c>
       <c r="B80" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C80" t="s" s="0">
+        <v>167</v>
+      </c>
+      <c r="D80" t="s" s="0">
+        <v>168</v>
+      </c>
+      <c r="E80" t="s" s="0">
+        <v>228</v>
+      </c>
+      <c r="F80" t="s" s="0">
         <v>162</v>
       </c>
-      <c r="C80" t="s" s="0">
-        <v>169</v>
-      </c>
-      <c r="D80" t="s" s="0">
-        <v>170</v>
-      </c>
-      <c r="E80" t="s" s="0">
-        <v>230</v>
-      </c>
-      <c r="F80" t="s" s="0">
-        <v>164</v>
-      </c>
       <c r="G80" t="s" s="0">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="81">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A81" t="s" s="0">
         <v>18</v>
       </c>
       <c r="B81" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C81" t="s" s="0">
+        <v>171</v>
+      </c>
+      <c r="D81" t="s" s="0">
+        <v>172</v>
+      </c>
+      <c r="E81" t="s" s="0">
+        <v>230</v>
+      </c>
+      <c r="F81" t="s" s="0">
         <v>162</v>
       </c>
-      <c r="C81" t="s" s="0">
-        <v>173</v>
-      </c>
-      <c r="D81" t="s" s="0">
-        <v>174</v>
-      </c>
-      <c r="E81" t="s" s="0">
-        <v>232</v>
-      </c>
-      <c r="F81" t="s" s="0">
-        <v>164</v>
-      </c>
       <c r="G81" t="s" s="0">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="82">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A82" t="s" s="0">
         <v>18</v>
       </c>
       <c r="B82" t="s" s="0">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="C82" t="s" s="0">
         <v>3</v>
@@ -3577,10 +3797,10 @@
         <v>4</v>
       </c>
       <c r="G82" t="s" s="0">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="83">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A83" t="s" s="0">
         <v>18</v>
       </c>
@@ -3588,7 +3808,7 @@
         <v>1</v>
       </c>
       <c r="C83" t="s" s="0">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="D83" t="s" s="0">
         <v>3</v>
@@ -3600,7 +3820,467 @@
         <v>4</v>
       </c>
       <c r="G83" t="s" s="0">
-        <v>239</v>
+        <v>237</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A84" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B84" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C84" t="s" s="0">
+        <v>164</v>
+      </c>
+      <c r="D84" t="s" s="0">
+        <v>168</v>
+      </c>
+      <c r="E84" t="s" s="0">
+        <v>221</v>
+      </c>
+      <c r="F84" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G84" t="s" s="0">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A85" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B85" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C85" t="s" s="0">
+        <v>188</v>
+      </c>
+      <c r="D85" t="s" s="0">
+        <v>223</v>
+      </c>
+      <c r="E85" t="s" s="0">
+        <v>224</v>
+      </c>
+      <c r="F85" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G85" t="s" s="0">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A86" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B86" t="s" s="0">
+        <v>249</v>
+      </c>
+      <c r="C86" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="D86" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E86" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F86" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="G86" t="s" s="0">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A87" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B87" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C87" t="s" s="0">
+        <v>251</v>
+      </c>
+      <c r="D87" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E87" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F87" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="G87" t="s" s="0">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A88" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B88" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C88" t="s" s="0">
+        <v>253</v>
+      </c>
+      <c r="D88" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E88" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F88" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="G88" t="s" s="0">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="B89" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C89" t="s" s="0">
+        <v>177</v>
+      </c>
+      <c r="D89" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="E89" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="F89" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G89" t="s" s="0">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="B90" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C90" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="D90" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="E90" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="F90" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G90" t="s" s="0">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="B91" t="s" s="0">
+        <v>249</v>
+      </c>
+      <c r="C91" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="D91" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E91" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F91" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="G91" t="s" s="0">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="B92" t="s" s="0">
+        <v>236</v>
+      </c>
+      <c r="C92" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="D92" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E92" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F92" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G92" t="s" s="0">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="B93" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="D93" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E93" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F93" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G93" t="s" s="0">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B94" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C94" t="s" s="0">
+        <v>164</v>
+      </c>
+      <c r="D94" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="E94" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="F94" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G94" t="s" s="0">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B95" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C95" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="D95" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="E95" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="F95" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G95" t="s" s="0">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B96" t="s" s="0">
+        <v>249</v>
+      </c>
+      <c r="C96" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="D96" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E96" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F96" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="G96" t="s" s="0">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B97" t="s" s="0">
+        <v>236</v>
+      </c>
+      <c r="C97" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="D97" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E97" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F97" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G97" t="s" s="0">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B98" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C98" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="D98" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E98" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F98" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G98" t="s" s="0">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B99" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C99" t="s" s="0">
+        <v>167</v>
+      </c>
+      <c r="D99" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="E99" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="F99" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G99" t="s" s="0">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B100" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C100" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="D100" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="E100" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="F100" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G100" t="s" s="0">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B101" t="s" s="0">
+        <v>249</v>
+      </c>
+      <c r="C101" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="D101" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E101" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F101" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="G101" t="s" s="0">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B102" t="s" s="0">
+        <v>236</v>
+      </c>
+      <c r="C102" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="D102" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E102" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F102" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G102" t="s" s="0">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B103" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C103" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="D103" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E103" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F103" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G103" t="s" s="0">
+        <v>268</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
improvised POM structure by separating base page and base test
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1023" uniqueCount="290">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1079" uniqueCount="297">
   <si>
     <t>extractCategoryCatalog</t>
   </si>
@@ -1192,6 +1192,45 @@
   </si>
   <si>
     <t>2026-07-23 18:44:21</t>
+  </si>
+  <si>
+    <t>stale element reference: stale element not found in the current frame
+  (Session info: chrome=150.0.7871.47)
+For documentation on this error, please visit: https://www.selenium.dev/documentation/webdriver/troubleshooting/errors#stale-element-reference-exception
+Build info: version: '4.21.0', revision: '79ed462ef4'
+System info: os.name: 'Windows 11', os.arch: 'amd64', os.version: '10.0', java.version: '21.0.10'
+Driver info: org.openqa.selenium.chrome.ChromeDriver
+Command: [67a854d01c4003a4f5944fd9f86775ed, isElementDisplayed {id=f.5B4CBD3216A188CB8A12625D7E03650C.d.59E7493151B423DFC710FDCB05D907C6.e.1697}]
+Capabilities {acceptInsecureCerts: false, browserName: chrome, browserVersion: 150.0.7871.47, chrome: {chromedriverVersion: 150.0.7871.124 (9261fd0a595..., userDataDir: C:\Users\2506400\AppData\Lo...}, fedcm:accounts: true, goog:chromeOptions: {debuggerAddress: localhost:55535}, goog:processID: 25760, networkConnectionEnabled: false, pageLoadStrategy: normal, platformName: windows, proxy: Proxy(), se:cdp: ws://localhost:55535/devtoo..., se:cdpVersion: 150.0.7871.47, setWindowRect: true, strictFileInteractability: false, timeouts: {implicit: 0, pageLoad: 300000, script: 30000}, unhandledPromptBehavior: dismiss and notify, webauthn:extension:credBlob: true, webauthn:extension:largeBlob: true, webauthn:extension:minPinLength: true, webauthn:extension:prf: true, webauthn:virtualAuthenticators: true}
+Element: [[ChromeDriver: chrome on windows (67a854d01c4003a4f5944fd9f86775ed)] -&gt; xpath: //div[contains(@class,'card--white')]]
+Session ID: 67a854d01c4003a4f5944fd9f86775ed</t>
+  </si>
+  <si>
+    <t>2026-07-23 19:43:32</t>
+  </si>
+  <si>
+    <t>stale element reference: stale element not found in the current frame
+  (Session info: chrome=150.0.7871.47)
+For documentation on this error, please visit: https://www.selenium.dev/documentation/webdriver/troubleshooting/errors#stale-element-reference-exception
+Build info: version: '4.21.0', revision: '79ed462ef4'
+System info: os.name: 'Windows 11', os.arch: 'amd64', os.version: '10.0', java.version: '21.0.10'
+Driver info: org.openqa.selenium.chrome.ChromeDriver
+Command: [ecd22cd6a781d5c71bdf92d1acba74cd, isElementDisplayed {id=f.BDCA8E81CF035C786D0E40226717BBB9.d.CA4255D9BDD09D2BB86CEC09E6B6F3B5.e.1713}]
+Capabilities {acceptInsecureCerts: false, browserName: chrome, browserVersion: 150.0.7871.47, chrome: {chromedriverVersion: 150.0.7871.124 (9261fd0a595..., userDataDir: C:\Users\2506400\AppData\Lo...}, fedcm:accounts: true, goog:chromeOptions: {debuggerAddress: localhost:53529}, goog:processID: 29588, networkConnectionEnabled: false, pageLoadStrategy: normal, platformName: windows, proxy: Proxy(), se:cdp: ws://localhost:53529/devtoo..., se:cdpVersion: 150.0.7871.47, setWindowRect: true, strictFileInteractability: false, timeouts: {implicit: 0, pageLoad: 300000, script: 30000}, unhandledPromptBehavior: dismiss and notify, webauthn:extension:credBlob: true, webauthn:extension:largeBlob: true, webauthn:extension:minPinLength: true, webauthn:extension:prf: true, webauthn:virtualAuthenticators: true}
+Element: [[ChromeDriver: chrome on windows (ecd22cd6a781d5c71bdf92d1acba74cd)] -&gt; xpath: //div[contains(@class,'card--white')]]
+Session ID: ecd22cd6a781d5c71bdf92d1acba74cd</t>
+  </si>
+  <si>
+    <t>2026-07-23 19:44:13</t>
+  </si>
+  <si>
+    <t>2026-07-23 19:44:52</t>
+  </si>
+  <si>
+    <t>2026-07-23 19:45:35</t>
+  </si>
+  <si>
+    <t>2026-07-23 19:46:15</t>
   </si>
 </sst>
 </file>
@@ -1807,7 +1846,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88BFA3FA-6A41-46D8-9F46-57C4912E9286}">
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="14.08984375"/>
@@ -2095,6 +2134,29 @@
         <v>235</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>231</v>
+      </c>
+      <c r="C13" t="s" s="0">
+        <v>232</v>
+      </c>
+      <c r="D13" t="s" s="0">
+        <v>215</v>
+      </c>
+      <c r="E13" t="s" s="0">
+        <v>233</v>
+      </c>
+      <c r="F13" t="s" s="0">
+        <v>234</v>
+      </c>
+      <c r="G13" t="s" s="0">
+        <v>235</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2102,7 +2164,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G125"/>
+  <dimension ref="A1:G132"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" customWidth="true" width="12.0"/>
@@ -4988,6 +5050,167 @@
         <v>289</v>
       </c>
     </row>
+    <row r="126">
+      <c r="A126" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="B126" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C126" t="s" s="0">
+        <v>290</v>
+      </c>
+      <c r="D126" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E126" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F126" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="G126" t="s" s="0">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B127" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C127" t="s" s="0">
+        <v>292</v>
+      </c>
+      <c r="D127" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E127" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F127" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="G127" t="s" s="0">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B128" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C128" t="s" s="0">
+        <v>167</v>
+      </c>
+      <c r="D128" t="s" s="0">
+        <v>168</v>
+      </c>
+      <c r="E128" t="s" s="0">
+        <v>228</v>
+      </c>
+      <c r="F128" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G128" t="s" s="0">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B129" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C129" t="s" s="0">
+        <v>171</v>
+      </c>
+      <c r="D129" t="s" s="0">
+        <v>172</v>
+      </c>
+      <c r="E129" t="s" s="0">
+        <v>230</v>
+      </c>
+      <c r="F129" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G129" t="s" s="0">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B130" t="s" s="0">
+        <v>249</v>
+      </c>
+      <c r="C130" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="D130" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E130" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F130" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="G130" t="s" s="0">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B131" t="s" s="0">
+        <v>236</v>
+      </c>
+      <c r="C131" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="D131" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E131" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F131" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G131" t="s" s="0">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B132" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C132" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="D132" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E132" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F132" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G132" t="s" s="0">
+        <v>296</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix stale element exception for dynamic element caused due to page factory
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2506400\Desktop\Pooja-Workspace\AlisonAutomation\src\test\resources\"/>
     </mc:Choice>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="84">
   <si>
     <t>TC_01</t>
   </si>
@@ -230,12 +230,63 @@
   </si>
   <si>
     <t>aisha.khanna@techsolutions.com</t>
+  </si>
+  <si>
+    <t>Python for Data Science: From the Basics to Advanced</t>
+  </si>
+  <si>
+    <t>Python is one of the best and fastest-growing programming languages used in data analysis worldwide. This free online course shows you how to apply the fundamental programming concepts of Python such as looping, variables, data types and data structures to data science. It also explores the NumPy and Pandas libraries that will help you further manipulate, analyze and visualize data in Python.</t>
+  </si>
+  <si>
+    <t>6-10
+Avg. Hours</t>
+  </si>
+  <si>
+    <t>20,033</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>Ermin Dedic</t>
+  </si>
+  <si>
+    <t>Diploma in E-Commerce Web Development</t>
+  </si>
+  <si>
+    <t>This diploma course teaches you how to develop a website to successfully drive e-commerce. We explain how to build an e-commerce website from scratch using HTML, CSS, Javascript, PHP and SQL. We then show you how to develop advanced e-commerce functionalities to display products online, using simple and effective CSS, PHP and SQL code in any development environment. This course can also help small businesses widen their customer base and grow.</t>
+  </si>
+  <si>
+    <t>133,738</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>ClayDesk E-Learning</t>
+  </si>
+  <si>
+    <t>Advanced Diploma in Python Programming for the Novice to Expert</t>
+  </si>
+  <si>
+    <t>Python is a popular programming language because it is fast, versatile and easy to understand. This free online Python course will hone your passion for programming by taking you through the fundamentals and more advanced features of Python. You will learn exactly how Python programming works, the different applications that Python can work for such as software development and mathematical computations and which areas you can apply them in.</t>
+  </si>
+  <si>
+    <t>15-20
+Avg. Hours</t>
+  </si>
+  <si>
+    <t>36,036</t>
+  </si>
+  <si>
+    <t>Juan Galvan</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -615,20 +666,20 @@
   <dimension ref="A1:P4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="22" customWidth="1"/>
-    <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="22.6328125" customWidth="1"/>
-    <col min="8" max="8" width="28.26953125" customWidth="1"/>
-    <col min="9" max="9" width="10.81640625" customWidth="1"/>
-    <col min="10" max="10" width="24.90625" customWidth="1"/>
-    <col min="11" max="11" width="20.6328125" customWidth="1"/>
-    <col min="12" max="12" width="21.81640625" customWidth="1"/>
-    <col min="13" max="14" width="15.7265625" customWidth="1"/>
-    <col min="15" max="15" width="59.6328125" customWidth="1"/>
-    <col min="16" max="16" width="30.1796875" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="12.0"/>
+    <col min="2" max="2" customWidth="true" width="22.0"/>
+    <col min="3" max="3" customWidth="true" width="14.0"/>
+    <col min="4" max="4" customWidth="true" width="16.0"/>
+    <col min="5" max="6" customWidth="true" width="14.0"/>
+    <col min="7" max="7" customWidth="true" width="22.6328125"/>
+    <col min="8" max="8" customWidth="true" width="28.26953125"/>
+    <col min="9" max="9" customWidth="true" width="10.81640625"/>
+    <col min="10" max="10" customWidth="true" width="24.90625"/>
+    <col min="11" max="11" customWidth="true" width="20.6328125"/>
+    <col min="12" max="12" customWidth="true" width="21.81640625"/>
+    <col min="13" max="14" customWidth="true" width="15.7265625"/>
+    <col min="15" max="15" customWidth="true" width="59.6328125"/>
+    <col min="16" max="16" customWidth="true" width="30.1796875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.35">
@@ -703,28 +754,28 @@
       <c r="G2" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" t="s" s="0">
         <v>31</v>
       </c>
-      <c r="I2" t="s">
+      <c r="I2" t="s" s="0">
         <v>32</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" t="s" s="0">
         <v>33</v>
       </c>
       <c r="K2" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="L2" t="s">
+      <c r="L2" t="s" s="0">
         <v>55</v>
       </c>
-      <c r="M2" t="s">
+      <c r="M2" t="s" s="0">
         <v>60</v>
       </c>
-      <c r="N2" t="s">
+      <c r="N2" t="s" s="0">
         <v>34</v>
       </c>
-      <c r="O2" t="s">
+      <c r="O2" t="s" s="0">
         <v>35</v>
       </c>
       <c r="P2" s="5" t="s">
@@ -753,28 +804,28 @@
       <c r="G3" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H3" t="s" s="0">
         <v>50</v>
       </c>
-      <c r="I3" t="s">
+      <c r="I3" t="s" s="0">
         <v>38</v>
       </c>
-      <c r="J3" t="s">
+      <c r="J3" t="s" s="0">
         <v>51</v>
       </c>
       <c r="K3" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="L3" t="s">
+      <c r="L3" t="s" s="0">
         <v>54</v>
       </c>
-      <c r="M3" t="s">
+      <c r="M3" t="s" s="0">
         <v>59</v>
       </c>
-      <c r="N3" t="s">
+      <c r="N3" t="s" s="0">
         <v>37</v>
       </c>
-      <c r="O3" t="s">
+      <c r="O3" t="s" s="0">
         <v>36</v>
       </c>
       <c r="P3" s="5" t="s">
@@ -803,10 +854,10 @@
       <c r="G4" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="H4" t="s">
+      <c r="H4" t="s" s="0">
         <v>58</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" t="s" s="0">
         <v>48</v>
       </c>
       <c r="J4" s="2" t="s">
@@ -815,16 +866,16 @@
       <c r="K4" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="L4" t="s">
+      <c r="L4" t="s" s="0">
         <v>56</v>
       </c>
-      <c r="M4" t="s">
+      <c r="M4" t="s" s="0">
         <v>61</v>
       </c>
-      <c r="N4" t="s">
+      <c r="N4" t="s" s="0">
         <v>39</v>
       </c>
-      <c r="O4" t="s">
+      <c r="O4" t="s" s="0">
         <v>40</v>
       </c>
       <c r="P4" s="5" t="s">
@@ -844,16 +895,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88BFA3FA-6A41-46D8-9F46-57C4912E9286}">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.08984375" customWidth="1"/>
-    <col min="2" max="2" width="37.54296875" customWidth="1"/>
-    <col min="3" max="3" width="30.453125" customWidth="1"/>
-    <col min="4" max="4" width="18.7265625" customWidth="1"/>
-    <col min="5" max="5" width="17.7265625" customWidth="1"/>
-    <col min="6" max="6" width="14.54296875" customWidth="1"/>
-    <col min="7" max="7" width="15.7265625" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="14.08984375"/>
+    <col min="2" max="2" customWidth="true" width="37.54296875"/>
+    <col min="3" max="3" customWidth="true" width="30.453125"/>
+    <col min="4" max="4" customWidth="true" width="18.7265625"/>
+    <col min="5" max="5" customWidth="true" width="17.7265625"/>
+    <col min="6" max="6" customWidth="true" width="14.54296875"/>
+    <col min="7" max="7" customWidth="true" width="15.7265625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
@@ -879,6 +930,98 @@
         <v>27</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>68</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>69</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>70</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>71</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>72</v>
+      </c>
+      <c r="G2" t="s" s="0">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>74</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>75</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>70</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>76</v>
+      </c>
+      <c r="F3" t="s" s="0">
+        <v>77</v>
+      </c>
+      <c r="G3" t="s" s="0">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>80</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>81</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>82</v>
+      </c>
+      <c r="F4" t="s" s="0">
+        <v>77</v>
+      </c>
+      <c r="G4" t="s" s="0">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>2</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>68</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>69</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>70</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>71</v>
+      </c>
+      <c r="F5" t="s" s="0">
+        <v>72</v>
+      </c>
+      <c r="G5" t="s" s="0">
+        <v>73</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
fix search result page
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="87">
   <si>
     <t>TC_01</t>
   </si>
@@ -280,6 +280,15 @@
   </si>
   <si>
     <t>Juan Galvan</t>
+  </si>
+  <si>
+    <t>20,035</t>
+  </si>
+  <si>
+    <t>133,906</t>
+  </si>
+  <si>
+    <t>36,059</t>
   </si>
 </sst>
 </file>
@@ -895,7 +904,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88BFA3FA-6A41-46D8-9F46-57C4912E9286}">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="14.08984375"/>
@@ -1022,6 +1031,144 @@
         <v>73</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>74</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>75</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>70</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>76</v>
+      </c>
+      <c r="F6" t="s" s="0">
+        <v>77</v>
+      </c>
+      <c r="G6" t="s" s="0">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>2</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>68</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>69</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>70</v>
+      </c>
+      <c r="E7" t="s" s="0">
+        <v>84</v>
+      </c>
+      <c r="F7" t="s" s="0">
+        <v>72</v>
+      </c>
+      <c r="G7" t="s" s="0">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>2</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>68</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>69</v>
+      </c>
+      <c r="D8" t="s" s="0">
+        <v>70</v>
+      </c>
+      <c r="E8" t="s" s="0">
+        <v>84</v>
+      </c>
+      <c r="F8" t="s" s="0">
+        <v>72</v>
+      </c>
+      <c r="G8" t="s" s="0">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>74</v>
+      </c>
+      <c r="C9" t="s" s="0">
+        <v>75</v>
+      </c>
+      <c r="D9" t="s" s="0">
+        <v>70</v>
+      </c>
+      <c r="E9" t="s" s="0">
+        <v>85</v>
+      </c>
+      <c r="F9" t="s" s="0">
+        <v>77</v>
+      </c>
+      <c r="G9" t="s" s="0">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="C10" t="s" s="0">
+        <v>80</v>
+      </c>
+      <c r="D10" t="s" s="0">
+        <v>81</v>
+      </c>
+      <c r="E10" t="s" s="0">
+        <v>86</v>
+      </c>
+      <c r="F10" t="s" s="0">
+        <v>77</v>
+      </c>
+      <c r="G10" t="s" s="0">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>2</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>68</v>
+      </c>
+      <c r="C11" t="s" s="0">
+        <v>69</v>
+      </c>
+      <c r="D11" t="s" s="0">
+        <v>70</v>
+      </c>
+      <c r="E11" t="s" s="0">
+        <v>84</v>
+      </c>
+      <c r="F11" t="s" s="0">
+        <v>72</v>
+      </c>
+      <c r="G11" t="s" s="0">
+        <v>73</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
optimised driver usage in TestListener
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="89">
   <si>
     <t>TC_01</t>
   </si>
@@ -289,6 +289,12 @@
   </si>
   <si>
     <t>36,059</t>
+  </si>
+  <si>
+    <t>36,066</t>
+  </si>
+  <si>
+    <t>20,042</t>
   </si>
 </sst>
 </file>
@@ -904,7 +910,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88BFA3FA-6A41-46D8-9F46-57C4912E9286}">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="14.08984375"/>
@@ -1169,6 +1175,121 @@
         <v>73</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>74</v>
+      </c>
+      <c r="C12" t="s" s="0">
+        <v>75</v>
+      </c>
+      <c r="D12" t="s" s="0">
+        <v>70</v>
+      </c>
+      <c r="E12" t="s" s="0">
+        <v>85</v>
+      </c>
+      <c r="F12" t="s" s="0">
+        <v>77</v>
+      </c>
+      <c r="G12" t="s" s="0">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="C13" t="s" s="0">
+        <v>80</v>
+      </c>
+      <c r="D13" t="s" s="0">
+        <v>81</v>
+      </c>
+      <c r="E13" t="s" s="0">
+        <v>86</v>
+      </c>
+      <c r="F13" t="s" s="0">
+        <v>77</v>
+      </c>
+      <c r="G13" t="s" s="0">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="0">
+        <v>2</v>
+      </c>
+      <c r="B14" t="s" s="0">
+        <v>68</v>
+      </c>
+      <c r="C14" t="s" s="0">
+        <v>69</v>
+      </c>
+      <c r="D14" t="s" s="0">
+        <v>70</v>
+      </c>
+      <c r="E14" t="s" s="0">
+        <v>84</v>
+      </c>
+      <c r="F14" t="s" s="0">
+        <v>72</v>
+      </c>
+      <c r="G14" t="s" s="0">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="B15" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="C15" t="s" s="0">
+        <v>80</v>
+      </c>
+      <c r="D15" t="s" s="0">
+        <v>81</v>
+      </c>
+      <c r="E15" t="s" s="0">
+        <v>87</v>
+      </c>
+      <c r="F15" t="s" s="0">
+        <v>77</v>
+      </c>
+      <c r="G15" t="s" s="0">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s" s="0">
+        <v>2</v>
+      </c>
+      <c r="B16" t="s" s="0">
+        <v>68</v>
+      </c>
+      <c r="C16" t="s" s="0">
+        <v>69</v>
+      </c>
+      <c r="D16" t="s" s="0">
+        <v>70</v>
+      </c>
+      <c r="E16" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="F16" t="s" s="0">
+        <v>72</v>
+      </c>
+      <c r="G16" t="s" s="0">
+        <v>73</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
simplified search filter funtionality
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="95">
   <si>
     <t>TC_01</t>
   </si>
@@ -295,6 +295,24 @@
   </si>
   <si>
     <t>20,042</t>
+  </si>
+  <si>
+    <t>134,005</t>
+  </si>
+  <si>
+    <t>36,078</t>
+  </si>
+  <si>
+    <t>20,068</t>
+  </si>
+  <si>
+    <t>134,114</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>0</t>
   </si>
 </sst>
 </file>
@@ -910,7 +928,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88BFA3FA-6A41-46D8-9F46-57C4912E9286}">
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="14.08984375"/>
@@ -1290,6 +1308,351 @@
         <v>73</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B17" t="s" s="0">
+        <v>74</v>
+      </c>
+      <c r="C17" t="s" s="0">
+        <v>75</v>
+      </c>
+      <c r="D17" t="s" s="0">
+        <v>70</v>
+      </c>
+      <c r="E17" t="s" s="0">
+        <v>89</v>
+      </c>
+      <c r="F17" t="s" s="0">
+        <v>77</v>
+      </c>
+      <c r="G17" t="s" s="0">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="B18" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="C18" t="s" s="0">
+        <v>80</v>
+      </c>
+      <c r="D18" t="s" s="0">
+        <v>81</v>
+      </c>
+      <c r="E18" t="s" s="0">
+        <v>87</v>
+      </c>
+      <c r="F18" t="s" s="0">
+        <v>77</v>
+      </c>
+      <c r="G18" t="s" s="0">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s" s="0">
+        <v>2</v>
+      </c>
+      <c r="B19" t="s" s="0">
+        <v>68</v>
+      </c>
+      <c r="C19" t="s" s="0">
+        <v>69</v>
+      </c>
+      <c r="D19" t="s" s="0">
+        <v>70</v>
+      </c>
+      <c r="E19" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="F19" t="s" s="0">
+        <v>72</v>
+      </c>
+      <c r="G19" t="s" s="0">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B20" t="s" s="0">
+        <v>74</v>
+      </c>
+      <c r="C20" t="s" s="0">
+        <v>75</v>
+      </c>
+      <c r="D20" t="s" s="0">
+        <v>70</v>
+      </c>
+      <c r="E20" t="s" s="0">
+        <v>89</v>
+      </c>
+      <c r="F20" t="s" s="0">
+        <v>77</v>
+      </c>
+      <c r="G20" t="s" s="0">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="B21" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="C21" t="s" s="0">
+        <v>80</v>
+      </c>
+      <c r="D21" t="s" s="0">
+        <v>81</v>
+      </c>
+      <c r="E21" t="s" s="0">
+        <v>87</v>
+      </c>
+      <c r="F21" t="s" s="0">
+        <v>77</v>
+      </c>
+      <c r="G21" t="s" s="0">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s" s="0">
+        <v>2</v>
+      </c>
+      <c r="B22" t="s" s="0">
+        <v>68</v>
+      </c>
+      <c r="C22" t="s" s="0">
+        <v>69</v>
+      </c>
+      <c r="D22" t="s" s="0">
+        <v>70</v>
+      </c>
+      <c r="E22" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="F22" t="s" s="0">
+        <v>72</v>
+      </c>
+      <c r="G22" t="s" s="0">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="B23" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="C23" t="s" s="0">
+        <v>80</v>
+      </c>
+      <c r="D23" t="s" s="0">
+        <v>81</v>
+      </c>
+      <c r="E23" t="s" s="0">
+        <v>90</v>
+      </c>
+      <c r="F23" t="s" s="0">
+        <v>77</v>
+      </c>
+      <c r="G23" t="s" s="0">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s" s="0">
+        <v>2</v>
+      </c>
+      <c r="B24" t="s" s="0">
+        <v>68</v>
+      </c>
+      <c r="C24" t="s" s="0">
+        <v>69</v>
+      </c>
+      <c r="D24" t="s" s="0">
+        <v>70</v>
+      </c>
+      <c r="E24" t="s" s="0">
+        <v>91</v>
+      </c>
+      <c r="F24" t="s" s="0">
+        <v>72</v>
+      </c>
+      <c r="G24" t="s" s="0">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B25" t="s" s="0">
+        <v>74</v>
+      </c>
+      <c r="C25" t="s" s="0">
+        <v>75</v>
+      </c>
+      <c r="D25" t="s" s="0">
+        <v>70</v>
+      </c>
+      <c r="E25" t="s" s="0">
+        <v>92</v>
+      </c>
+      <c r="F25" t="s" s="0">
+        <v>77</v>
+      </c>
+      <c r="G25" t="s" s="0">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s" s="0">
+        <v>2</v>
+      </c>
+      <c r="B26" t="s" s="0">
+        <v>68</v>
+      </c>
+      <c r="C26" t="s" s="0">
+        <v>69</v>
+      </c>
+      <c r="D26" t="s" s="0">
+        <v>70</v>
+      </c>
+      <c r="E26" t="s" s="0">
+        <v>91</v>
+      </c>
+      <c r="F26" t="s" s="0">
+        <v>72</v>
+      </c>
+      <c r="G26" t="s" s="0">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s" s="0">
+        <v>2</v>
+      </c>
+      <c r="B27" t="s" s="0">
+        <v>68</v>
+      </c>
+      <c r="C27" t="s" s="0">
+        <v>69</v>
+      </c>
+      <c r="D27" t="s" s="0">
+        <v>70</v>
+      </c>
+      <c r="E27" t="s" s="0">
+        <v>91</v>
+      </c>
+      <c r="F27" t="s" s="0">
+        <v>72</v>
+      </c>
+      <c r="G27" t="s" s="0">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B28" t="s" s="0">
+        <v>93</v>
+      </c>
+      <c r="C28" t="s" s="0">
+        <v>93</v>
+      </c>
+      <c r="D28" t="s" s="0">
+        <v>93</v>
+      </c>
+      <c r="E28" t="s" s="0">
+        <v>93</v>
+      </c>
+      <c r="F28" t="s" s="0">
+        <v>94</v>
+      </c>
+      <c r="G28" t="s" s="0">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B29" t="s" s="0">
+        <v>74</v>
+      </c>
+      <c r="C29" t="s" s="0">
+        <v>75</v>
+      </c>
+      <c r="D29" t="s" s="0">
+        <v>70</v>
+      </c>
+      <c r="E29" t="s" s="0">
+        <v>92</v>
+      </c>
+      <c r="F29" t="s" s="0">
+        <v>77</v>
+      </c>
+      <c r="G29" t="s" s="0">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="B30" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="C30" t="s" s="0">
+        <v>80</v>
+      </c>
+      <c r="D30" t="s" s="0">
+        <v>81</v>
+      </c>
+      <c r="E30" t="s" s="0">
+        <v>90</v>
+      </c>
+      <c r="F30" t="s" s="0">
+        <v>77</v>
+      </c>
+      <c r="G30" t="s" s="0">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s" s="0">
+        <v>2</v>
+      </c>
+      <c r="B31" t="s" s="0">
+        <v>68</v>
+      </c>
+      <c r="C31" t="s" s="0">
+        <v>69</v>
+      </c>
+      <c r="D31" t="s" s="0">
+        <v>70</v>
+      </c>
+      <c r="E31" t="s" s="0">
+        <v>91</v>
+      </c>
+      <c r="F31" t="s" s="0">
+        <v>72</v>
+      </c>
+      <c r="G31" t="s" s="0">
+        <v>73</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
fix stale element exception
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="98">
   <si>
     <t>TC_01</t>
   </si>
@@ -313,6 +313,15 @@
   </si>
   <si>
     <t>0</t>
+  </si>
+  <si>
+    <t>134,221</t>
+  </si>
+  <si>
+    <t>36,080</t>
+  </si>
+  <si>
+    <t>20,079</t>
   </si>
 </sst>
 </file>
@@ -928,7 +937,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88BFA3FA-6A41-46D8-9F46-57C4912E9286}">
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="14.08984375"/>
@@ -1653,6 +1662,167 @@
         <v>73</v>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="s" s="0">
+        <v>2</v>
+      </c>
+      <c r="B32" t="s" s="0">
+        <v>68</v>
+      </c>
+      <c r="C32" t="s" s="0">
+        <v>69</v>
+      </c>
+      <c r="D32" t="s" s="0">
+        <v>70</v>
+      </c>
+      <c r="E32" t="s" s="0">
+        <v>91</v>
+      </c>
+      <c r="F32" t="s" s="0">
+        <v>72</v>
+      </c>
+      <c r="G32" t="s" s="0">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B33" t="s" s="0">
+        <v>74</v>
+      </c>
+      <c r="C33" t="s" s="0">
+        <v>75</v>
+      </c>
+      <c r="D33" t="s" s="0">
+        <v>70</v>
+      </c>
+      <c r="E33" t="s" s="0">
+        <v>92</v>
+      </c>
+      <c r="F33" t="s" s="0">
+        <v>77</v>
+      </c>
+      <c r="G33" t="s" s="0">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="B34" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="C34" t="s" s="0">
+        <v>80</v>
+      </c>
+      <c r="D34" t="s" s="0">
+        <v>81</v>
+      </c>
+      <c r="E34" t="s" s="0">
+        <v>90</v>
+      </c>
+      <c r="F34" t="s" s="0">
+        <v>77</v>
+      </c>
+      <c r="G34" t="s" s="0">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s" s="0">
+        <v>2</v>
+      </c>
+      <c r="B35" t="s" s="0">
+        <v>68</v>
+      </c>
+      <c r="C35" t="s" s="0">
+        <v>69</v>
+      </c>
+      <c r="D35" t="s" s="0">
+        <v>70</v>
+      </c>
+      <c r="E35" t="s" s="0">
+        <v>91</v>
+      </c>
+      <c r="F35" t="s" s="0">
+        <v>72</v>
+      </c>
+      <c r="G35" t="s" s="0">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B36" t="s" s="0">
+        <v>74</v>
+      </c>
+      <c r="C36" t="s" s="0">
+        <v>75</v>
+      </c>
+      <c r="D36" t="s" s="0">
+        <v>70</v>
+      </c>
+      <c r="E36" t="s" s="0">
+        <v>95</v>
+      </c>
+      <c r="F36" t="s" s="0">
+        <v>77</v>
+      </c>
+      <c r="G36" t="s" s="0">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="B37" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="C37" t="s" s="0">
+        <v>80</v>
+      </c>
+      <c r="D37" t="s" s="0">
+        <v>81</v>
+      </c>
+      <c r="E37" t="s" s="0">
+        <v>96</v>
+      </c>
+      <c r="F37" t="s" s="0">
+        <v>77</v>
+      </c>
+      <c r="G37" t="s" s="0">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s" s="0">
+        <v>2</v>
+      </c>
+      <c r="B38" t="s" s="0">
+        <v>68</v>
+      </c>
+      <c r="C38" t="s" s="0">
+        <v>69</v>
+      </c>
+      <c r="D38" t="s" s="0">
+        <v>70</v>
+      </c>
+      <c r="E38" t="s" s="0">
+        <v>97</v>
+      </c>
+      <c r="F38" t="s" s="0">
+        <v>72</v>
+      </c>
+      <c r="G38" t="s" s="0">
+        <v>73</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>